<commit_message>
3.4.8: kernel-size vs params plot
</commit_message>
<xml_diff>
--- a/datasets/sgt_files/InVitroBioFilm_SGT_scaling.xlsx
+++ b/datasets/sgt_files/InVitroBioFilm_SGT_scaling.xlsx
@@ -440,25 +440,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C2">
-        <v>1.12989675044522</v>
+        <v>1.3</v>
       </c>
       <c r="D2">
-        <v>0.113967</v>
+        <v>0.223665</v>
       </c>
       <c r="E2">
-        <v>0.0111726845525644</v>
+        <v>0.08689313063566455</v>
       </c>
       <c r="F2">
-        <v>1.08278537031645</v>
+        <v>1.05307844348342</v>
       </c>
       <c r="G2">
-        <v>-0.9432208836866045</v>
+        <v>-0.6504019707362143</v>
       </c>
       <c r="H2">
-        <v>-0.928579184308906</v>
+        <v>-0.7360841467267152</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -466,25 +466,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="C3">
-        <v>1.796601730428249</v>
+        <v>3.0840089349921</v>
       </c>
       <c r="D3">
-        <v>0.039636</v>
+        <v>0.047857</v>
       </c>
       <c r="E3">
-        <v>0.002826119915675514</v>
+        <v>0.005268825939218126</v>
       </c>
       <c r="F3">
-        <v>1.59659709562646</v>
+        <v>1.591064607026499</v>
       </c>
       <c r="G3">
-        <v>-1.401910180260961</v>
+        <v>-1.320054529380785</v>
       </c>
       <c r="H3">
-        <v>-1.410745692789158</v>
+        <v>-1.299983122420791</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -492,25 +492,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>80.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C4">
-        <v>3.572891763761611</v>
+        <v>2.478574859336174</v>
       </c>
       <c r="D4">
-        <v>0.019578</v>
+        <v>0.01952</v>
       </c>
       <c r="E4">
-        <v>0.001783419810987369</v>
+        <v>0.001232376205187</v>
       </c>
       <c r="F4">
-        <v>1.903632516084238</v>
+        <v>1.898176483497676</v>
       </c>
       <c r="G4">
-        <v>-1.708231675828481</v>
+        <v>-1.709520186669327</v>
       </c>
       <c r="H4">
-        <v>-1.698871069010518</v>
+        <v>-1.621887446920606</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -518,25 +518,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>137.2</v>
+        <v>130.9</v>
       </c>
       <c r="C5">
-        <v>4.304519588628781</v>
+        <v>4.787599723359411</v>
       </c>
       <c r="D5">
-        <v>0.012534</v>
+        <v>0.012653</v>
       </c>
       <c r="E5">
-        <v>0.0009046155721262668</v>
+        <v>0.001167132335636747</v>
       </c>
       <c r="F5">
-        <v>2.137354111370733</v>
+        <v>2.116939646550756</v>
       </c>
       <c r="G5">
-        <v>-1.901910309636048</v>
+        <v>-1.897806491960256</v>
       </c>
       <c r="H5">
-        <v>-1.918197954724794</v>
+        <v>-1.851187625856062</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -544,25 +544,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>203.4</v>
+        <v>214.1</v>
       </c>
       <c r="C6">
-        <v>4.77772609791171</v>
+        <v>4.670117771534247</v>
       </c>
       <c r="D6">
-        <v>0.008934000000000001</v>
+        <v>0.007606</v>
       </c>
       <c r="E6">
-        <v>0.000431483745026649</v>
+        <v>0.000416579190817571</v>
       </c>
       <c r="F6">
-        <v>2.308350948586726</v>
+        <v>2.330616667294438</v>
       </c>
       <c r="G6">
-        <v>-2.04895405186418</v>
+        <v>-2.118843678924436</v>
       </c>
       <c r="H6">
-        <v>-2.07866324560903</v>
+        <v>-2.075156681738808</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -570,25 +570,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>290.4</v>
+        <v>288.1</v>
       </c>
       <c r="C7">
-        <v>4.742713709821976</v>
+        <v>5.685165882462103</v>
       </c>
       <c r="D7">
-        <v>0.005514</v>
+        <v>0.00615</v>
       </c>
       <c r="E7">
-        <v>0.0003042593922589372</v>
+        <v>0.0003635351121663185</v>
       </c>
       <c r="F7">
-        <v>2.462996612028056</v>
+        <v>2.459543258280413</v>
       </c>
       <c r="G7">
-        <v>-2.258533238230245</v>
+        <v>-2.211124884224583</v>
       </c>
       <c r="H7">
-        <v>-2.22378441727581</v>
+        <v>-2.210293191789403</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -596,25 +596,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>397.9</v>
+        <v>394</v>
       </c>
       <c r="C8">
-        <v>4.958606435055898</v>
+        <v>3.346640106136302</v>
       </c>
       <c r="D8">
-        <v>0.004329999999999999</v>
+        <v>0.004235000000000001</v>
       </c>
       <c r="E8">
-        <v>0.0001732114956410868</v>
+        <v>0.0001603347193287288</v>
       </c>
       <c r="F8">
-        <v>2.599773939146388</v>
+        <v>2.595496221825574</v>
       </c>
       <c r="G8">
-        <v>-2.363512103646635</v>
+        <v>-2.373146585333274</v>
       </c>
       <c r="H8">
-        <v>-2.352137747897287</v>
+        <v>-2.352794508887963</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -622,25 +622,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.9</v>
+        <v>515.2</v>
       </c>
       <c r="C9">
-        <v>5.700779673771728</v>
+        <v>3.805843460317889</v>
       </c>
       <c r="D9">
-        <v>0.003257</v>
+        <v>0.003294</v>
       </c>
       <c r="E9">
-        <v>0.0001395711686241507</v>
+        <v>0.0001124000790826136</v>
       </c>
       <c r="F9">
-        <v>2.712565527873308</v>
+        <v>2.711975854351756</v>
       </c>
       <c r="G9">
-        <v>-2.487182241435127</v>
+        <v>-2.482276405166265</v>
       </c>
       <c r="H9">
-        <v>-2.457982600872541</v>
+        <v>-2.474884536330605</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -648,25 +648,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>667</v>
+        <v>662.5</v>
       </c>
       <c r="C10">
-        <v>4.695151163109069</v>
+        <v>6.057593948462082</v>
       </c>
       <c r="D10">
-        <v>0.002504999999999999</v>
+        <v>0.002638000000000001</v>
       </c>
       <c r="E10">
-        <v>7.528095524249295E-05</v>
+        <v>7.209253313161726E-05</v>
       </c>
       <c r="F10">
-        <v>2.824125833916549</v>
+        <v>2.821185882608845</v>
       </c>
       <c r="G10">
-        <v>-2.601192269796736</v>
+        <v>-2.578725208789654</v>
       </c>
       <c r="H10">
-        <v>-2.56267200479263</v>
+        <v>-2.589354809439706</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -674,25 +674,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="C11">
-        <v>8.364275886836296</v>
+        <v>9.599131905195039</v>
       </c>
       <c r="D11">
-        <v>0.002171</v>
+        <v>0.00213</v>
       </c>
       <c r="E11">
-        <v>6.04510821518799E-05</v>
+        <v>6.881537295950343E-05</v>
       </c>
       <c r="F11">
-        <v>2.909288524162251</v>
+        <v>2.910037123553051</v>
       </c>
       <c r="G11">
-        <v>-2.66334017654558</v>
+        <v>-2.671620396561262</v>
       </c>
       <c r="H11">
-        <v>-2.642589599089996</v>
+        <v>-2.68248568743035</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -718,7 +718,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.441950929022662</v>
+        <v>-2.457595894667791</v>
       </c>
     </row>
   </sheetData>
@@ -741,290 +741,290 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="B2">
-        <v>0.114118894657337</v>
+        <v>0.2234229411226657</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>20.17474747474747</v>
+        <v>19.3969696969697</v>
       </c>
       <c r="B3">
-        <v>0.07153840198621657</v>
+        <v>0.1156212373834673</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>28.24949494949495</v>
+        <v>27.4939393939394</v>
       </c>
       <c r="B4">
-        <v>0.05259964516128546</v>
+        <v>0.07556595810281702</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>36.32424242424242</v>
+        <v>35.59090909090909</v>
       </c>
       <c r="B5">
-        <v>0.04180625295572488</v>
+        <v>0.05516354196624016</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>44.3989898989899</v>
+        <v>43.68787878787879</v>
       </c>
       <c r="B6">
-        <v>0.03480208572938091</v>
+        <v>0.04296524975839557</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>52.47373737373737</v>
+        <v>51.78484848484848</v>
       </c>
       <c r="B7">
-        <v>0.02987537705570119</v>
+        <v>0.03492127028347099</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>60.54848484848484</v>
+        <v>59.88181818181819</v>
       </c>
       <c r="B8">
-        <v>0.02621373526820083</v>
+        <v>0.02925286548600948</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>68.62323232323232</v>
+        <v>67.97878787878788</v>
       </c>
       <c r="B9">
-        <v>0.02338103360402072</v>
+        <v>0.02506208489084306</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.69797979797978</v>
+        <v>76.07575757575758</v>
       </c>
       <c r="B10">
-        <v>0.02112174936903392</v>
+        <v>0.02184900993129131</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.77272727272725</v>
+        <v>84.17272727272727</v>
       </c>
       <c r="B11">
-        <v>0.01927604335909764</v>
+        <v>0.01931428318245793</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.84747474747473</v>
+        <v>92.26969696969697</v>
       </c>
       <c r="B12">
-        <v>0.01773870091217781</v>
+        <v>0.01726822968450587</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.9222222222222</v>
+        <v>100.3666666666667</v>
       </c>
       <c r="B13">
-        <v>0.01643757540808223</v>
+        <v>0.01558512248656729</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.9969696969697</v>
+        <v>108.4636363636364</v>
       </c>
       <c r="B14">
-        <v>0.01532150915408134</v>
+        <v>0.01417848879016148</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>117.0717171717172</v>
+        <v>116.5606060606061</v>
       </c>
       <c r="B15">
-        <v>0.01435319723341663</v>
+        <v>0.01298699511530168</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>125.1464646464646</v>
+        <v>124.6575757575758</v>
       </c>
       <c r="B16">
-        <v>0.0135047825124472</v>
+        <v>0.01196599002919759</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>133.2212121212121</v>
+        <v>132.7545454545455</v>
       </c>
       <c r="B17">
-        <v>0.01275503402534345</v>
+        <v>0.0110822316650582</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>141.2959595959596</v>
+        <v>140.8515151515152</v>
       </c>
       <c r="B18">
-        <v>0.01208748145851442</v>
+        <v>0.01031048744007662</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>149.3707070707071</v>
+        <v>148.9484848484849</v>
       </c>
       <c r="B19">
-        <v>0.01148914749613198</v>
+        <v>0.009631275999786809</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.4454545454545</v>
+        <v>157.0454545454546</v>
       </c>
       <c r="B20">
-        <v>0.01094966553484734</v>
+        <v>0.009029328839544866</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.520202020202</v>
+        <v>165.1424242424243</v>
       </c>
       <c r="B21">
-        <v>0.01046065249826879</v>
+        <v>0.008492518339989152</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.5949494949495</v>
+        <v>173.2393939393939</v>
       </c>
       <c r="B22">
-        <v>0.01001525453838841</v>
+        <v>0.008011095705198019</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.6696969696969</v>
+        <v>181.3363636363637</v>
       </c>
       <c r="B23">
-        <v>0.009607812388484292</v>
+        <v>0.007577139428687919</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.7444444444444</v>
+        <v>189.4333333333334</v>
       </c>
       <c r="B24">
-        <v>0.009233611095551531</v>
+        <v>0.007184149648374311</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.8191919191919</v>
+        <v>197.5303030303031</v>
       </c>
       <c r="B25">
-        <v>0.008888690275485224</v>
+        <v>0.006826745424516108</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.8939393939393</v>
+        <v>205.6272727272728</v>
       </c>
       <c r="B26">
-        <v>0.00856969845168928</v>
+        <v>0.006500435816382649</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.9686868686868</v>
+        <v>213.7242424242424</v>
       </c>
       <c r="B27">
-        <v>0.008273779955781664</v>
+        <v>0.006201444662158525</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>222.0434343434343</v>
+        <v>221.8212121212121</v>
       </c>
       <c r="B28">
-        <v>0.007998486190224757</v>
+        <v>0.005926574970018011</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>230.1181818181818</v>
+        <v>229.9181818181818</v>
       </c>
       <c r="B29">
-        <v>0.007741705333417221</v>
+        <v>0.00567310289062023</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.1929292929293</v>
+        <v>238.0151515151516</v>
       </c>
       <c r="B30">
-        <v>0.007501606158254927</v>
+        <v>0.005438694034608454</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.2676767676767</v>
+        <v>246.1121212121213</v>
       </c>
       <c r="B31">
-        <v>0.007276592760105602</v>
+        <v>0.00522133684803717</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.3424242424242</v>
+        <v>254.2090909090909</v>
       </c>
       <c r="B32">
-        <v>0.007065267796277352</v>
+        <v>0.005019289137692525</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.4171717171717</v>
+        <v>262.3060606060606</v>
       </c>
       <c r="B33">
-        <v>0.006866402423782412</v>
+        <v>0.004831034826267896</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4919191919192</v>
+        <v>270.4030303030303</v>
       </c>
       <c r="B34">
-        <v>0.006678911551119365</v>
+        <v>0.0046552487335509</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5666666666667</v>
+        <v>278.5000000000001</v>
       </c>
       <c r="B35">
-        <v>0.006501833337750171</v>
+        <v>0.004490767704652825</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.6414141414141</v>
+        <v>286.5969696969697</v>
       </c>
       <c r="B36">
-        <v>0.006334312112962199</v>
+        <v>0.004336566794921568</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.7161616161616</v>
+        <v>294.6939393939394</v>
       </c>
       <c r="B37">
-        <v>0.006175584065620148</v>
+        <v>0.004191739511663775</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -1032,511 +1032,511 @@
         <v>302.7909090909091</v>
       </c>
       <c r="B38">
-        <v>0.006024965193333106</v>
+        <v>0.004055481331892936</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8656565656565</v>
+        <v>310.8878787878788</v>
       </c>
       <c r="B39">
-        <v>0.005881841104820782</v>
+        <v>0.003927075881962371</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.940404040404</v>
+        <v>318.9848484848485</v>
       </c>
       <c r="B40">
-        <v>0.005745658350741072</v>
+        <v>0.003805883292700867</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0151515151515</v>
+        <v>327.0818181818182</v>
       </c>
       <c r="B41">
-        <v>0.005615917021766245</v>
+        <v>0.003691330342352621</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.089898989899</v>
+        <v>335.1787878787879</v>
       </c>
       <c r="B42">
-        <v>0.005492164402560705</v>
+        <v>0.00358290207638999</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.1646464646465</v>
+        <v>343.2757575757576</v>
       </c>
       <c r="B43">
-        <v>0.005373989509709177</v>
+        <v>0.003480134653385886</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.2393939393939</v>
+        <v>351.3727272727273</v>
       </c>
       <c r="B44">
-        <v>0.005261018372958773</v>
+        <v>0.003382609213512734</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.3141414141414</v>
+        <v>359.469696969697</v>
       </c>
       <c r="B45">
-        <v>0.005152909944174143</v>
+        <v>0.003289946603801274</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.3888888888889</v>
+        <v>367.5666666666667</v>
       </c>
       <c r="B46">
-        <v>0.005049352538531013</v>
+        <v>0.003201802824248834</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.4636363636363</v>
+        <v>375.6636363636364</v>
       </c>
       <c r="B47">
-        <v>0.004950060728737752</v>
+        <v>0.003117865082885064</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.5383838383838</v>
+        <v>383.7606060606061</v>
       </c>
       <c r="B48">
-        <v>0.004854772626283929</v>
+        <v>0.003037848367260696</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.6131313131313</v>
+        <v>391.8575757575758</v>
       </c>
       <c r="B49">
-        <v>0.004763247494494139</v>
+        <v>0.002961492455503649</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.6878787878787</v>
+        <v>399.9545454545455</v>
       </c>
       <c r="B50">
-        <v>0.004675263647001852</v>
+        <v>0.002888559302845906</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>407.7626262626262</v>
+        <v>408.0515151515152</v>
       </c>
       <c r="B51">
-        <v>0.004590616592533375</v>
+        <v>0.002818830749954937</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>415.8373737373737</v>
+        <v>416.1484848484849</v>
       </c>
       <c r="B52">
-        <v>0.004509117392907075</v>
+        <v>0.002752106507966855</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>423.9121212121212</v>
+        <v>424.2454545454546</v>
       </c>
       <c r="B53">
-        <v>0.004430591206145848</v>
+        <v>0.002688202382178486</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>431.9868686868687</v>
+        <v>432.3424242424243</v>
       </c>
       <c r="B54">
-        <v>0.004354875990761184</v>
+        <v>0.002626948702199065</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.0616161616161</v>
+        <v>440.439393939394</v>
       </c>
       <c r="B55">
-        <v>0.004281821350746441</v>
+        <v>0.002568188931217557</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.1363636363636</v>
+        <v>448.5363636363637</v>
       </c>
       <c r="B56">
-        <v>0.004211287503737038</v>
+        <v>0.00251177843109041</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.2111111111111</v>
+        <v>456.6333333333334</v>
       </c>
       <c r="B57">
-        <v>0.00414314435725427</v>
+        <v>0.002457583363342884</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.2858585858585</v>
+        <v>464.7303030303031</v>
       </c>
       <c r="B58">
-        <v>0.00407727068002698</v>
+        <v>0.002405479709022215</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.360606060606</v>
+        <v>472.8272727272728</v>
       </c>
       <c r="B59">
-        <v>0.004013553357146009</v>
+        <v>0.002355352392737675</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.4353535353535</v>
+        <v>480.9242424242425</v>
       </c>
       <c r="B60">
-        <v>0.003951886719303136</v>
+        <v>0.002307094498248114</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>488.510101010101</v>
+        <v>489.0212121212122</v>
       </c>
       <c r="B61">
-        <v>0.003892171937642248</v>
+        <v>0.00226060656467445</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>496.5848484848485</v>
+        <v>497.1181818181819</v>
       </c>
       <c r="B62">
-        <v>0.003834316476841483</v>
+        <v>0.00221579595387411</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>504.6595959595959</v>
+        <v>505.2151515151515</v>
       </c>
       <c r="B63">
-        <v>0.003778233599980349</v>
+        <v>0.002172576280758743</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>512.7343434343434</v>
+        <v>513.3121212121213</v>
       </c>
       <c r="B64">
-        <v>0.003723841919549707</v>
+        <v>0.002130866899400167</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>520.8090909090909</v>
+        <v>521.4090909090909</v>
       </c>
       <c r="B65">
-        <v>0.003671064989655256</v>
+        <v>0.00209059243868117</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>528.8838383838383</v>
+        <v>529.5060606060606</v>
       </c>
       <c r="B66">
-        <v>0.003619830935063521</v>
+        <v>0.002051682382031121</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>536.9585858585858</v>
+        <v>537.6030303030303</v>
       </c>
       <c r="B67">
-        <v>0.003570072113257467</v>
+        <v>0.002014070686461129</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.0333333333333</v>
+        <v>545.7</v>
       </c>
       <c r="B68">
-        <v>0.003521724806118537</v>
+        <v>0.001977695436696093</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.1080808080808</v>
+        <v>553.7969696969697</v>
       </c>
       <c r="B69">
-        <v>0.003474728938243024</v>
+        <v>0.001942498530705191</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.1828282828283</v>
+        <v>561.8939393939394</v>
       </c>
       <c r="B70">
-        <v>0.003429027819241569</v>
+        <v>0.001908425393369704</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.2575757575758</v>
+        <v>569.9909090909091</v>
       </c>
       <c r="B71">
-        <v>0.003384567907668399</v>
+        <v>0.001875424715407219</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>577.3323232323232</v>
+        <v>578.0878787878788</v>
       </c>
       <c r="B72">
-        <v>0.003341298594487549</v>
+        <v>0.001843448215002397</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>585.4070707070706</v>
+        <v>586.1848484848484</v>
       </c>
       <c r="B73">
-        <v>0.00329917200421184</v>
+        <v>0.001812450419883519</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>593.4818181818181</v>
+        <v>594.2818181818182</v>
       </c>
       <c r="B74">
-        <v>0.003258142812051314</v>
+        <v>0.001782388467836827</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>601.5565656565656</v>
+        <v>602.3787878787879</v>
       </c>
       <c r="B75">
-        <v>0.003218168075584502</v>
+        <v>0.001753221923872184</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>609.631313131313</v>
+        <v>610.4757575757576</v>
       </c>
       <c r="B76">
-        <v>0.003179207079621927</v>
+        <v>0.001724912612448014</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>617.7060606060605</v>
+        <v>618.5727272727273</v>
       </c>
       <c r="B77">
-        <v>0.003141221193068869</v>
+        <v>0.001697424463334556</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>625.780808080808</v>
+        <v>626.6696969696969</v>
       </c>
       <c r="B78">
-        <v>0.003104173736716384</v>
+        <v>0.00167072336984511</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>633.8555555555555</v>
+        <v>634.7666666666667</v>
       </c>
       <c r="B79">
-        <v>0.003068029860997553</v>
+        <v>0.00164477705829798</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>641.930303030303</v>
+        <v>642.8636363636364</v>
       </c>
       <c r="B80">
-        <v>0.003032756432841862</v>
+        <v>0.001619554967689372</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.0050505050505</v>
+        <v>650.9606060606061</v>
       </c>
       <c r="B81">
-        <v>0.002998321930845916</v>
+        <v>0.001595028138661609</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>658.0797979797979</v>
+        <v>659.0575757575757</v>
       </c>
       <c r="B82">
-        <v>0.002964696348054624</v>
+        <v>0.001571169110943376</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>666.1545454545454</v>
+        <v>667.1545454545454</v>
       </c>
       <c r="B83">
-        <v>0.002931851101714743</v>
+        <v>0.001547951828520692</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>674.2292929292929</v>
+        <v>675.2515151515152</v>
       </c>
       <c r="B84">
-        <v>0.002899758949423204</v>
+        <v>0.001525351551870314</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>682.3040404040404</v>
+        <v>683.3484848484849</v>
       </c>
       <c r="B85">
-        <v>0.002868393911146696</v>
+        <v>0.001503344776652226</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>690.3787878787878</v>
+        <v>691.4454545454546</v>
       </c>
       <c r="B86">
-        <v>0.002837731196637552</v>
+        <v>0.001481909158315892</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>698.4535353535352</v>
+        <v>699.5424242424242</v>
       </c>
       <c r="B87">
-        <v>0.002807747137814382</v>
+        <v>0.001461023442126762</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>706.5282828282827</v>
+        <v>707.6393939393939</v>
       </c>
       <c r="B88">
-        <v>0.002778419125714995</v>
+        <v>0.001440667398165869</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>714.6030303030302</v>
+        <v>715.7363636363636</v>
       </c>
       <c r="B89">
-        <v>0.002749725551664224</v>
+        <v>0.001420821760896863</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>722.6777777777777</v>
+        <v>723.8333333333334</v>
       </c>
       <c r="B90">
-        <v>0.002721645752330935</v>
+        <v>0.001401468172932123</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>730.7525252525252</v>
+        <v>731.9303030303031</v>
       </c>
       <c r="B91">
-        <v>0.00269415995837694</v>
+        <v>0.001382589132662983</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>738.8272727272727</v>
+        <v>740.0272727272727</v>
       </c>
       <c r="B92">
-        <v>0.002667249246426297</v>
+        <v>0.001364167945449245</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>746.9020202020201</v>
+        <v>748.1242424242424</v>
       </c>
       <c r="B93">
-        <v>0.00264089549410671</v>
+        <v>0.001346188678090202</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>754.9767676767676</v>
+        <v>756.2212121212121</v>
       </c>
       <c r="B94">
-        <v>0.002615081337935753</v>
+        <v>0.001328636116323822</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>763.0515151515151</v>
+        <v>764.3181818181819</v>
       </c>
       <c r="B95">
-        <v>0.002589790133843706</v>
+        <v>0.001311495725122791</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>771.1262626262626</v>
+        <v>772.4151515151515</v>
       </c>
       <c r="B96">
-        <v>0.002565005920142038</v>
+        <v>0.00129475361157598</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>779.2010101010101</v>
+        <v>780.5121212121212</v>
       </c>
       <c r="B97">
-        <v>0.002540713382762229</v>
+        <v>0.001278396490161965</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>787.2757575757574</v>
+        <v>788.6090909090909</v>
       </c>
       <c r="B98">
-        <v>0.002516897822603894</v>
+        <v>0.001262411650237472</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>795.3505050505049</v>
+        <v>796.7060606060606</v>
       </c>
       <c r="B99">
-        <v>0.002493545124844073</v>
+        <v>0.001246786925578432</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>803.4252525252524</v>
+        <v>804.8030303030304</v>
       </c>
       <c r="B100">
-        <v>0.002470641730071381</v>
+        <v>0.001231510665824734</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="B101">
-        <v>0.002448174607119392</v>
+        <v>0.001216571709691934</v>
       </c>
     </row>
   </sheetData>
@@ -1580,25 +1580,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C2">
-        <v>1.12989675044522</v>
+        <v>1.3</v>
       </c>
       <c r="D2">
-        <v>0.113967</v>
+        <v>0.223665</v>
       </c>
       <c r="E2">
-        <v>0.0111726845525644</v>
+        <v>0.08689313063566455</v>
       </c>
       <c r="F2">
-        <v>1.08278537031645</v>
+        <v>1.05307844348342</v>
       </c>
       <c r="G2">
-        <v>-0.9432208836866045</v>
+        <v>-0.6504019707362143</v>
       </c>
       <c r="H2">
-        <v>-0.928579184308906</v>
+        <v>-0.7360841467267152</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1606,25 +1606,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="C3">
-        <v>1.796601730428249</v>
+        <v>3.0840089349921</v>
       </c>
       <c r="D3">
-        <v>0.039636</v>
+        <v>0.047857</v>
       </c>
       <c r="E3">
-        <v>0.002826119915675514</v>
+        <v>0.005268825939218126</v>
       </c>
       <c r="F3">
-        <v>1.59659709562646</v>
+        <v>1.591064607026499</v>
       </c>
       <c r="G3">
-        <v>-1.401910180260961</v>
+        <v>-1.320054529380785</v>
       </c>
       <c r="H3">
-        <v>-1.410745692789158</v>
+        <v>-1.299983122420791</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1632,25 +1632,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>80.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C4">
-        <v>3.572891763761611</v>
+        <v>2.478574859336174</v>
       </c>
       <c r="D4">
-        <v>0.019578</v>
+        <v>0.01952</v>
       </c>
       <c r="E4">
-        <v>0.001783419810987369</v>
+        <v>0.001232376205187</v>
       </c>
       <c r="F4">
-        <v>1.903632516084238</v>
+        <v>1.898176483497676</v>
       </c>
       <c r="G4">
-        <v>-1.708231675828481</v>
+        <v>-1.709520186669327</v>
       </c>
       <c r="H4">
-        <v>-1.698871069010518</v>
+        <v>-1.621887446920606</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1658,25 +1658,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>137.2</v>
+        <v>130.9</v>
       </c>
       <c r="C5">
-        <v>4.304519588628781</v>
+        <v>4.787599723359411</v>
       </c>
       <c r="D5">
-        <v>0.012534</v>
+        <v>0.012653</v>
       </c>
       <c r="E5">
-        <v>0.0009046155721262668</v>
+        <v>0.001167132335636747</v>
       </c>
       <c r="F5">
-        <v>2.137354111370733</v>
+        <v>2.116939646550756</v>
       </c>
       <c r="G5">
-        <v>-1.901910309636048</v>
+        <v>-1.897806491960256</v>
       </c>
       <c r="H5">
-        <v>-1.918197954724794</v>
+        <v>-1.851187625856062</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1684,25 +1684,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>203.4</v>
+        <v>214.1</v>
       </c>
       <c r="C6">
-        <v>4.77772609791171</v>
+        <v>4.670117771534247</v>
       </c>
       <c r="D6">
-        <v>0.008934000000000001</v>
+        <v>0.007606</v>
       </c>
       <c r="E6">
-        <v>0.000431483745026649</v>
+        <v>0.000416579190817571</v>
       </c>
       <c r="F6">
-        <v>2.308350948586726</v>
+        <v>2.330616667294438</v>
       </c>
       <c r="G6">
-        <v>-2.04895405186418</v>
+        <v>-2.118843678924436</v>
       </c>
       <c r="H6">
-        <v>-2.07866324560903</v>
+        <v>-2.075156681738808</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1710,25 +1710,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>290.4</v>
+        <v>288.1</v>
       </c>
       <c r="C7">
-        <v>4.742713709821976</v>
+        <v>5.685165882462103</v>
       </c>
       <c r="D7">
-        <v>0.005514</v>
+        <v>0.00615</v>
       </c>
       <c r="E7">
-        <v>0.0003042593922589372</v>
+        <v>0.0003635351121663185</v>
       </c>
       <c r="F7">
-        <v>2.462996612028056</v>
+        <v>2.459543258280413</v>
       </c>
       <c r="G7">
-        <v>-2.258533238230245</v>
+        <v>-2.211124884224583</v>
       </c>
       <c r="H7">
-        <v>-2.22378441727581</v>
+        <v>-2.210293191789403</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1736,25 +1736,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>397.9</v>
+        <v>394</v>
       </c>
       <c r="C8">
-        <v>4.958606435055898</v>
+        <v>3.346640106136302</v>
       </c>
       <c r="D8">
-        <v>0.004329999999999999</v>
+        <v>0.004235000000000001</v>
       </c>
       <c r="E8">
-        <v>0.0001732114956410868</v>
+        <v>0.0001603347193287288</v>
       </c>
       <c r="F8">
-        <v>2.599773939146388</v>
+        <v>2.595496221825574</v>
       </c>
       <c r="G8">
-        <v>-2.363512103646635</v>
+        <v>-2.373146585333274</v>
       </c>
       <c r="H8">
-        <v>-2.352137747897287</v>
+        <v>-2.352794508887963</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1762,25 +1762,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.9</v>
+        <v>515.2</v>
       </c>
       <c r="C9">
-        <v>5.700779673771728</v>
+        <v>3.805843460317889</v>
       </c>
       <c r="D9">
-        <v>0.003257</v>
+        <v>0.003294</v>
       </c>
       <c r="E9">
-        <v>0.0001395711686241507</v>
+        <v>0.0001124000790826136</v>
       </c>
       <c r="F9">
-        <v>2.712565527873308</v>
+        <v>2.711975854351756</v>
       </c>
       <c r="G9">
-        <v>-2.487182241435127</v>
+        <v>-2.482276405166265</v>
       </c>
       <c r="H9">
-        <v>-2.457982600872541</v>
+        <v>-2.474884536330605</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1788,25 +1788,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>667</v>
+        <v>662.5</v>
       </c>
       <c r="C10">
-        <v>4.695151163109069</v>
+        <v>6.057593948462082</v>
       </c>
       <c r="D10">
-        <v>0.002504999999999999</v>
+        <v>0.002638000000000001</v>
       </c>
       <c r="E10">
-        <v>7.528095524249295E-05</v>
+        <v>7.209253313161726E-05</v>
       </c>
       <c r="F10">
-        <v>2.824125833916549</v>
+        <v>2.821185882608845</v>
       </c>
       <c r="G10">
-        <v>-2.601192269796736</v>
+        <v>-2.578725208789654</v>
       </c>
       <c r="H10">
-        <v>-2.56267200479263</v>
+        <v>-2.589354809439706</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1814,25 +1814,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="C11">
-        <v>8.364275886836296</v>
+        <v>9.599131905195039</v>
       </c>
       <c r="D11">
-        <v>0.002171</v>
+        <v>0.00213</v>
       </c>
       <c r="E11">
-        <v>6.04510821518799E-05</v>
+        <v>6.881537295950343E-05</v>
       </c>
       <c r="F11">
-        <v>2.909288524162251</v>
+        <v>2.910037123553051</v>
       </c>
       <c r="G11">
-        <v>-2.66334017654558</v>
+        <v>-2.671620396561262</v>
       </c>
       <c r="H11">
-        <v>-2.642589599089996</v>
+        <v>-2.68248568743035</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1858,7 +1858,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.441950929022662</v>
+        <v>-2.457595894667791</v>
       </c>
     </row>
   </sheetData>
@@ -1881,290 +1881,290 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="B2">
-        <v>0.114118894657337</v>
+        <v>0.2234229411226657</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>20.17474747474747</v>
+        <v>19.3969696969697</v>
       </c>
       <c r="B3">
-        <v>0.07153840198621657</v>
+        <v>0.1156212373834673</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>28.24949494949495</v>
+        <v>27.4939393939394</v>
       </c>
       <c r="B4">
-        <v>0.05259964516128546</v>
+        <v>0.07556595810281702</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>36.32424242424242</v>
+        <v>35.59090909090909</v>
       </c>
       <c r="B5">
-        <v>0.04180625295572488</v>
+        <v>0.05516354196624016</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>44.3989898989899</v>
+        <v>43.68787878787879</v>
       </c>
       <c r="B6">
-        <v>0.03480208572938091</v>
+        <v>0.04296524975839557</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>52.47373737373737</v>
+        <v>51.78484848484848</v>
       </c>
       <c r="B7">
-        <v>0.02987537705570119</v>
+        <v>0.03492127028347099</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>60.54848484848484</v>
+        <v>59.88181818181819</v>
       </c>
       <c r="B8">
-        <v>0.02621373526820083</v>
+        <v>0.02925286548600948</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>68.62323232323232</v>
+        <v>67.97878787878788</v>
       </c>
       <c r="B9">
-        <v>0.02338103360402072</v>
+        <v>0.02506208489084306</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.69797979797978</v>
+        <v>76.07575757575758</v>
       </c>
       <c r="B10">
-        <v>0.02112174936903392</v>
+        <v>0.02184900993129131</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.77272727272725</v>
+        <v>84.17272727272727</v>
       </c>
       <c r="B11">
-        <v>0.01927604335909764</v>
+        <v>0.01931428318245793</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.84747474747473</v>
+        <v>92.26969696969697</v>
       </c>
       <c r="B12">
-        <v>0.01773870091217781</v>
+        <v>0.01726822968450587</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.9222222222222</v>
+        <v>100.3666666666667</v>
       </c>
       <c r="B13">
-        <v>0.01643757540808223</v>
+        <v>0.01558512248656729</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.9969696969697</v>
+        <v>108.4636363636364</v>
       </c>
       <c r="B14">
-        <v>0.01532150915408134</v>
+        <v>0.01417848879016148</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>117.0717171717172</v>
+        <v>116.5606060606061</v>
       </c>
       <c r="B15">
-        <v>0.01435319723341663</v>
+        <v>0.01298699511530168</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>125.1464646464646</v>
+        <v>124.6575757575758</v>
       </c>
       <c r="B16">
-        <v>0.0135047825124472</v>
+        <v>0.01196599002919759</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>133.2212121212121</v>
+        <v>132.7545454545455</v>
       </c>
       <c r="B17">
-        <v>0.01275503402534345</v>
+        <v>0.0110822316650582</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>141.2959595959596</v>
+        <v>140.8515151515152</v>
       </c>
       <c r="B18">
-        <v>0.01208748145851442</v>
+        <v>0.01031048744007662</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>149.3707070707071</v>
+        <v>148.9484848484849</v>
       </c>
       <c r="B19">
-        <v>0.01148914749613198</v>
+        <v>0.009631275999786809</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.4454545454545</v>
+        <v>157.0454545454546</v>
       </c>
       <c r="B20">
-        <v>0.01094966553484734</v>
+        <v>0.009029328839544866</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.520202020202</v>
+        <v>165.1424242424243</v>
       </c>
       <c r="B21">
-        <v>0.01046065249826879</v>
+        <v>0.008492518339989152</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.5949494949495</v>
+        <v>173.2393939393939</v>
       </c>
       <c r="B22">
-        <v>0.01001525453838841</v>
+        <v>0.008011095705198019</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.6696969696969</v>
+        <v>181.3363636363637</v>
       </c>
       <c r="B23">
-        <v>0.009607812388484292</v>
+        <v>0.007577139428687919</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.7444444444444</v>
+        <v>189.4333333333334</v>
       </c>
       <c r="B24">
-        <v>0.009233611095551531</v>
+        <v>0.007184149648374311</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.8191919191919</v>
+        <v>197.5303030303031</v>
       </c>
       <c r="B25">
-        <v>0.008888690275485224</v>
+        <v>0.006826745424516108</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.8939393939393</v>
+        <v>205.6272727272728</v>
       </c>
       <c r="B26">
-        <v>0.00856969845168928</v>
+        <v>0.006500435816382649</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.9686868686868</v>
+        <v>213.7242424242424</v>
       </c>
       <c r="B27">
-        <v>0.008273779955781664</v>
+        <v>0.006201444662158525</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>222.0434343434343</v>
+        <v>221.8212121212121</v>
       </c>
       <c r="B28">
-        <v>0.007998486190224757</v>
+        <v>0.005926574970018011</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>230.1181818181818</v>
+        <v>229.9181818181818</v>
       </c>
       <c r="B29">
-        <v>0.007741705333417221</v>
+        <v>0.00567310289062023</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.1929292929293</v>
+        <v>238.0151515151516</v>
       </c>
       <c r="B30">
-        <v>0.007501606158254927</v>
+        <v>0.005438694034608454</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.2676767676767</v>
+        <v>246.1121212121213</v>
       </c>
       <c r="B31">
-        <v>0.007276592760105602</v>
+        <v>0.00522133684803717</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.3424242424242</v>
+        <v>254.2090909090909</v>
       </c>
       <c r="B32">
-        <v>0.007065267796277352</v>
+        <v>0.005019289137692525</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.4171717171717</v>
+        <v>262.3060606060606</v>
       </c>
       <c r="B33">
-        <v>0.006866402423782412</v>
+        <v>0.004831034826267896</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4919191919192</v>
+        <v>270.4030303030303</v>
       </c>
       <c r="B34">
-        <v>0.006678911551119365</v>
+        <v>0.0046552487335509</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5666666666667</v>
+        <v>278.5000000000001</v>
       </c>
       <c r="B35">
-        <v>0.006501833337750171</v>
+        <v>0.004490767704652825</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.6414141414141</v>
+        <v>286.5969696969697</v>
       </c>
       <c r="B36">
-        <v>0.006334312112962199</v>
+        <v>0.004336566794921568</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.7161616161616</v>
+        <v>294.6939393939394</v>
       </c>
       <c r="B37">
-        <v>0.006175584065620148</v>
+        <v>0.004191739511663775</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -2172,511 +2172,511 @@
         <v>302.7909090909091</v>
       </c>
       <c r="B38">
-        <v>0.006024965193333106</v>
+        <v>0.004055481331892936</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8656565656565</v>
+        <v>310.8878787878788</v>
       </c>
       <c r="B39">
-        <v>0.005881841104820782</v>
+        <v>0.003927075881962371</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.940404040404</v>
+        <v>318.9848484848485</v>
       </c>
       <c r="B40">
-        <v>0.005745658350741072</v>
+        <v>0.003805883292700867</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0151515151515</v>
+        <v>327.0818181818182</v>
       </c>
       <c r="B41">
-        <v>0.005615917021766245</v>
+        <v>0.003691330342352621</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.089898989899</v>
+        <v>335.1787878787879</v>
       </c>
       <c r="B42">
-        <v>0.005492164402560705</v>
+        <v>0.00358290207638999</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.1646464646465</v>
+        <v>343.2757575757576</v>
       </c>
       <c r="B43">
-        <v>0.005373989509709177</v>
+        <v>0.003480134653385886</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.2393939393939</v>
+        <v>351.3727272727273</v>
       </c>
       <c r="B44">
-        <v>0.005261018372958773</v>
+        <v>0.003382609213512734</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.3141414141414</v>
+        <v>359.469696969697</v>
       </c>
       <c r="B45">
-        <v>0.005152909944174143</v>
+        <v>0.003289946603801274</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.3888888888889</v>
+        <v>367.5666666666667</v>
       </c>
       <c r="B46">
-        <v>0.005049352538531013</v>
+        <v>0.003201802824248834</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.4636363636363</v>
+        <v>375.6636363636364</v>
       </c>
       <c r="B47">
-        <v>0.004950060728737752</v>
+        <v>0.003117865082885064</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.5383838383838</v>
+        <v>383.7606060606061</v>
       </c>
       <c r="B48">
-        <v>0.004854772626283929</v>
+        <v>0.003037848367260696</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.6131313131313</v>
+        <v>391.8575757575758</v>
       </c>
       <c r="B49">
-        <v>0.004763247494494139</v>
+        <v>0.002961492455503649</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.6878787878787</v>
+        <v>399.9545454545455</v>
       </c>
       <c r="B50">
-        <v>0.004675263647001852</v>
+        <v>0.002888559302845906</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>407.7626262626262</v>
+        <v>408.0515151515152</v>
       </c>
       <c r="B51">
-        <v>0.004590616592533375</v>
+        <v>0.002818830749954937</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>415.8373737373737</v>
+        <v>416.1484848484849</v>
       </c>
       <c r="B52">
-        <v>0.004509117392907075</v>
+        <v>0.002752106507966855</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>423.9121212121212</v>
+        <v>424.2454545454546</v>
       </c>
       <c r="B53">
-        <v>0.004430591206145848</v>
+        <v>0.002688202382178486</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>431.9868686868687</v>
+        <v>432.3424242424243</v>
       </c>
       <c r="B54">
-        <v>0.004354875990761184</v>
+        <v>0.002626948702199065</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.0616161616161</v>
+        <v>440.439393939394</v>
       </c>
       <c r="B55">
-        <v>0.004281821350746441</v>
+        <v>0.002568188931217557</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.1363636363636</v>
+        <v>448.5363636363637</v>
       </c>
       <c r="B56">
-        <v>0.004211287503737038</v>
+        <v>0.00251177843109041</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.2111111111111</v>
+        <v>456.6333333333334</v>
       </c>
       <c r="B57">
-        <v>0.00414314435725427</v>
+        <v>0.002457583363342884</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.2858585858585</v>
+        <v>464.7303030303031</v>
       </c>
       <c r="B58">
-        <v>0.00407727068002698</v>
+        <v>0.002405479709022215</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.360606060606</v>
+        <v>472.8272727272728</v>
       </c>
       <c r="B59">
-        <v>0.004013553357146009</v>
+        <v>0.002355352392737675</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.4353535353535</v>
+        <v>480.9242424242425</v>
       </c>
       <c r="B60">
-        <v>0.003951886719303136</v>
+        <v>0.002307094498248114</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>488.510101010101</v>
+        <v>489.0212121212122</v>
       </c>
       <c r="B61">
-        <v>0.003892171937642248</v>
+        <v>0.00226060656467445</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>496.5848484848485</v>
+        <v>497.1181818181819</v>
       </c>
       <c r="B62">
-        <v>0.003834316476841483</v>
+        <v>0.00221579595387411</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>504.6595959595959</v>
+        <v>505.2151515151515</v>
       </c>
       <c r="B63">
-        <v>0.003778233599980349</v>
+        <v>0.002172576280758743</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>512.7343434343434</v>
+        <v>513.3121212121213</v>
       </c>
       <c r="B64">
-        <v>0.003723841919549707</v>
+        <v>0.002130866899400167</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>520.8090909090909</v>
+        <v>521.4090909090909</v>
       </c>
       <c r="B65">
-        <v>0.003671064989655256</v>
+        <v>0.00209059243868117</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>528.8838383838383</v>
+        <v>529.5060606060606</v>
       </c>
       <c r="B66">
-        <v>0.003619830935063521</v>
+        <v>0.002051682382031121</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>536.9585858585858</v>
+        <v>537.6030303030303</v>
       </c>
       <c r="B67">
-        <v>0.003570072113257467</v>
+        <v>0.002014070686461129</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.0333333333333</v>
+        <v>545.7</v>
       </c>
       <c r="B68">
-        <v>0.003521724806118537</v>
+        <v>0.001977695436696093</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.1080808080808</v>
+        <v>553.7969696969697</v>
       </c>
       <c r="B69">
-        <v>0.003474728938243024</v>
+        <v>0.001942498530705191</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.1828282828283</v>
+        <v>561.8939393939394</v>
       </c>
       <c r="B70">
-        <v>0.003429027819241569</v>
+        <v>0.001908425393369704</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.2575757575758</v>
+        <v>569.9909090909091</v>
       </c>
       <c r="B71">
-        <v>0.003384567907668399</v>
+        <v>0.001875424715407219</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>577.3323232323232</v>
+        <v>578.0878787878788</v>
       </c>
       <c r="B72">
-        <v>0.003341298594487549</v>
+        <v>0.001843448215002397</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>585.4070707070706</v>
+        <v>586.1848484848484</v>
       </c>
       <c r="B73">
-        <v>0.00329917200421184</v>
+        <v>0.001812450419883519</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>593.4818181818181</v>
+        <v>594.2818181818182</v>
       </c>
       <c r="B74">
-        <v>0.003258142812051314</v>
+        <v>0.001782388467836827</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>601.5565656565656</v>
+        <v>602.3787878787879</v>
       </c>
       <c r="B75">
-        <v>0.003218168075584502</v>
+        <v>0.001753221923872184</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>609.631313131313</v>
+        <v>610.4757575757576</v>
       </c>
       <c r="B76">
-        <v>0.003179207079621927</v>
+        <v>0.001724912612448014</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>617.7060606060605</v>
+        <v>618.5727272727273</v>
       </c>
       <c r="B77">
-        <v>0.003141221193068869</v>
+        <v>0.001697424463334556</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>625.780808080808</v>
+        <v>626.6696969696969</v>
       </c>
       <c r="B78">
-        <v>0.003104173736716384</v>
+        <v>0.00167072336984511</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>633.8555555555555</v>
+        <v>634.7666666666667</v>
       </c>
       <c r="B79">
-        <v>0.003068029860997553</v>
+        <v>0.00164477705829798</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>641.930303030303</v>
+        <v>642.8636363636364</v>
       </c>
       <c r="B80">
-        <v>0.003032756432841862</v>
+        <v>0.001619554967689372</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.0050505050505</v>
+        <v>650.9606060606061</v>
       </c>
       <c r="B81">
-        <v>0.002998321930845916</v>
+        <v>0.001595028138661609</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>658.0797979797979</v>
+        <v>659.0575757575757</v>
       </c>
       <c r="B82">
-        <v>0.002964696348054624</v>
+        <v>0.001571169110943376</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>666.1545454545454</v>
+        <v>667.1545454545454</v>
       </c>
       <c r="B83">
-        <v>0.002931851101714743</v>
+        <v>0.001547951828520692</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>674.2292929292929</v>
+        <v>675.2515151515152</v>
       </c>
       <c r="B84">
-        <v>0.002899758949423204</v>
+        <v>0.001525351551870314</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>682.3040404040404</v>
+        <v>683.3484848484849</v>
       </c>
       <c r="B85">
-        <v>0.002868393911146696</v>
+        <v>0.001503344776652226</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>690.3787878787878</v>
+        <v>691.4454545454546</v>
       </c>
       <c r="B86">
-        <v>0.002837731196637552</v>
+        <v>0.001481909158315892</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>698.4535353535352</v>
+        <v>699.5424242424242</v>
       </c>
       <c r="B87">
-        <v>0.002807747137814382</v>
+        <v>0.001461023442126762</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>706.5282828282827</v>
+        <v>707.6393939393939</v>
       </c>
       <c r="B88">
-        <v>0.002778419125714995</v>
+        <v>0.001440667398165869</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>714.6030303030302</v>
+        <v>715.7363636363636</v>
       </c>
       <c r="B89">
-        <v>0.002749725551664224</v>
+        <v>0.001420821760896863</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>722.6777777777777</v>
+        <v>723.8333333333334</v>
       </c>
       <c r="B90">
-        <v>0.002721645752330935</v>
+        <v>0.001401468172932123</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>730.7525252525252</v>
+        <v>731.9303030303031</v>
       </c>
       <c r="B91">
-        <v>0.00269415995837694</v>
+        <v>0.001382589132662983</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>738.8272727272727</v>
+        <v>740.0272727272727</v>
       </c>
       <c r="B92">
-        <v>0.002667249246426297</v>
+        <v>0.001364167945449245</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>746.9020202020201</v>
+        <v>748.1242424242424</v>
       </c>
       <c r="B93">
-        <v>0.00264089549410671</v>
+        <v>0.001346188678090202</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>754.9767676767676</v>
+        <v>756.2212121212121</v>
       </c>
       <c r="B94">
-        <v>0.002615081337935753</v>
+        <v>0.001328636116323822</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>763.0515151515151</v>
+        <v>764.3181818181819</v>
       </c>
       <c r="B95">
-        <v>0.002589790133843706</v>
+        <v>0.001311495725122791</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>771.1262626262626</v>
+        <v>772.4151515151515</v>
       </c>
       <c r="B96">
-        <v>0.002565005920142038</v>
+        <v>0.00129475361157598</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>779.2010101010101</v>
+        <v>780.5121212121212</v>
       </c>
       <c r="B97">
-        <v>0.002540713382762229</v>
+        <v>0.001278396490161965</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>787.2757575757574</v>
+        <v>788.6090909090909</v>
       </c>
       <c r="B98">
-        <v>0.002516897822603894</v>
+        <v>0.001262411650237472</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>795.3505050505049</v>
+        <v>796.7060606060606</v>
       </c>
       <c r="B99">
-        <v>0.002493545124844073</v>
+        <v>0.001246786925578432</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>803.4252525252524</v>
+        <v>804.8030303030304</v>
       </c>
       <c r="B100">
-        <v>0.002470641730071381</v>
+        <v>0.001231510665824734</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="B101">
-        <v>0.002448174607119392</v>
+        <v>0.001216571709691934</v>
       </c>
     </row>
   </sheetData>
@@ -2720,25 +2720,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="C2">
-        <v>1.12989675044522</v>
+        <v>1.3</v>
       </c>
       <c r="D2">
-        <v>0.113967</v>
+        <v>0.223665</v>
       </c>
       <c r="E2">
-        <v>0.0111726845525644</v>
+        <v>0.08689313063566455</v>
       </c>
       <c r="F2">
-        <v>1.08278537031645</v>
+        <v>1.05307844348342</v>
       </c>
       <c r="G2">
-        <v>-0.9432208836866045</v>
+        <v>-0.6504019707362143</v>
       </c>
       <c r="H2">
-        <v>-0.928579184308906</v>
+        <v>-0.7360841467267152</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2746,25 +2746,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="C3">
-        <v>1.796601730428249</v>
+        <v>3.0840089349921</v>
       </c>
       <c r="D3">
-        <v>0.039636</v>
+        <v>0.047857</v>
       </c>
       <c r="E3">
-        <v>0.002826119915675514</v>
+        <v>0.005268825939218126</v>
       </c>
       <c r="F3">
-        <v>1.59659709562646</v>
+        <v>1.591064607026499</v>
       </c>
       <c r="G3">
-        <v>-1.401910180260961</v>
+        <v>-1.320054529380785</v>
       </c>
       <c r="H3">
-        <v>-1.410745692789158</v>
+        <v>-1.299983122420791</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2772,25 +2772,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>80.09999999999999</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="C4">
-        <v>3.572891763761611</v>
+        <v>2.478574859336174</v>
       </c>
       <c r="D4">
-        <v>0.019578</v>
+        <v>0.01952</v>
       </c>
       <c r="E4">
-        <v>0.001783419810987369</v>
+        <v>0.001232376205187</v>
       </c>
       <c r="F4">
-        <v>1.903632516084238</v>
+        <v>1.898176483497676</v>
       </c>
       <c r="G4">
-        <v>-1.708231675828481</v>
+        <v>-1.709520186669327</v>
       </c>
       <c r="H4">
-        <v>-1.698871069010518</v>
+        <v>-1.621887446920606</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2798,25 +2798,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>137.2</v>
+        <v>130.9</v>
       </c>
       <c r="C5">
-        <v>4.304519588628781</v>
+        <v>4.787599723359411</v>
       </c>
       <c r="D5">
-        <v>0.012534</v>
+        <v>0.012653</v>
       </c>
       <c r="E5">
-        <v>0.0009046155721262668</v>
+        <v>0.001167132335636747</v>
       </c>
       <c r="F5">
-        <v>2.137354111370733</v>
+        <v>2.116939646550756</v>
       </c>
       <c r="G5">
-        <v>-1.901910309636048</v>
+        <v>-1.897806491960256</v>
       </c>
       <c r="H5">
-        <v>-1.918197954724794</v>
+        <v>-1.851187625856062</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2824,25 +2824,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>203.4</v>
+        <v>214.1</v>
       </c>
       <c r="C6">
-        <v>4.77772609791171</v>
+        <v>4.670117771534247</v>
       </c>
       <c r="D6">
-        <v>0.008934000000000001</v>
+        <v>0.007606</v>
       </c>
       <c r="E6">
-        <v>0.000431483745026649</v>
+        <v>0.000416579190817571</v>
       </c>
       <c r="F6">
-        <v>2.308350948586726</v>
+        <v>2.330616667294438</v>
       </c>
       <c r="G6">
-        <v>-2.04895405186418</v>
+        <v>-2.118843678924436</v>
       </c>
       <c r="H6">
-        <v>-2.07866324560903</v>
+        <v>-2.075156681738808</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2850,25 +2850,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>290.4</v>
+        <v>288.1</v>
       </c>
       <c r="C7">
-        <v>4.742713709821976</v>
+        <v>5.685165882462103</v>
       </c>
       <c r="D7">
-        <v>0.005514</v>
+        <v>0.00615</v>
       </c>
       <c r="E7">
-        <v>0.0003042593922589372</v>
+        <v>0.0003635351121663185</v>
       </c>
       <c r="F7">
-        <v>2.462996612028056</v>
+        <v>2.459543258280413</v>
       </c>
       <c r="G7">
-        <v>-2.258533238230245</v>
+        <v>-2.211124884224583</v>
       </c>
       <c r="H7">
-        <v>-2.22378441727581</v>
+        <v>-2.210293191789403</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2876,25 +2876,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>397.9</v>
+        <v>394</v>
       </c>
       <c r="C8">
-        <v>4.958606435055898</v>
+        <v>3.346640106136302</v>
       </c>
       <c r="D8">
-        <v>0.004329999999999999</v>
+        <v>0.004235000000000001</v>
       </c>
       <c r="E8">
-        <v>0.0001732114956410868</v>
+        <v>0.0001603347193287288</v>
       </c>
       <c r="F8">
-        <v>2.599773939146388</v>
+        <v>2.595496221825574</v>
       </c>
       <c r="G8">
-        <v>-2.363512103646635</v>
+        <v>-2.373146585333274</v>
       </c>
       <c r="H8">
-        <v>-2.352137747897287</v>
+        <v>-2.352794508887963</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2902,25 +2902,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.9</v>
+        <v>515.2</v>
       </c>
       <c r="C9">
-        <v>5.700779673771728</v>
+        <v>3.805843460317889</v>
       </c>
       <c r="D9">
-        <v>0.003257</v>
+        <v>0.003294</v>
       </c>
       <c r="E9">
-        <v>0.0001395711686241507</v>
+        <v>0.0001124000790826136</v>
       </c>
       <c r="F9">
-        <v>2.712565527873308</v>
+        <v>2.711975854351756</v>
       </c>
       <c r="G9">
-        <v>-2.487182241435127</v>
+        <v>-2.482276405166265</v>
       </c>
       <c r="H9">
-        <v>-2.457982600872541</v>
+        <v>-2.474884536330605</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2928,25 +2928,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>667</v>
+        <v>662.5</v>
       </c>
       <c r="C10">
-        <v>4.695151163109069</v>
+        <v>6.057593948462082</v>
       </c>
       <c r="D10">
-        <v>0.002504999999999999</v>
+        <v>0.002638000000000001</v>
       </c>
       <c r="E10">
-        <v>7.528095524249295E-05</v>
+        <v>7.209253313161726E-05</v>
       </c>
       <c r="F10">
-        <v>2.824125833916549</v>
+        <v>2.821185882608845</v>
       </c>
       <c r="G10">
-        <v>-2.601192269796736</v>
+        <v>-2.578725208789654</v>
       </c>
       <c r="H10">
-        <v>-2.56267200479263</v>
+        <v>-2.589354809439706</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2954,25 +2954,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="C11">
-        <v>8.364275886836296</v>
+        <v>9.599131905195039</v>
       </c>
       <c r="D11">
-        <v>0.002171</v>
+        <v>0.00213</v>
       </c>
       <c r="E11">
-        <v>6.04510821518799E-05</v>
+        <v>6.881537295950343E-05</v>
       </c>
       <c r="F11">
-        <v>2.909288524162251</v>
+        <v>2.910037123553051</v>
       </c>
       <c r="G11">
-        <v>-2.66334017654558</v>
+        <v>-2.671620396561262</v>
       </c>
       <c r="H11">
-        <v>-2.642589599089996</v>
+        <v>-2.68248568743035</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2998,7 +2998,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.441950929022662</v>
+        <v>-2.457595894667791</v>
       </c>
     </row>
   </sheetData>
@@ -3021,290 +3021,290 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>12.1</v>
+        <v>11.3</v>
       </c>
       <c r="B2">
-        <v>0.114118894657337</v>
+        <v>0.2234229411226657</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>20.17474747474747</v>
+        <v>19.3969696969697</v>
       </c>
       <c r="B3">
-        <v>0.07153840198621657</v>
+        <v>0.1156212373834673</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>28.24949494949495</v>
+        <v>27.4939393939394</v>
       </c>
       <c r="B4">
-        <v>0.05259964516128546</v>
+        <v>0.07556595810281702</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>36.32424242424242</v>
+        <v>35.59090909090909</v>
       </c>
       <c r="B5">
-        <v>0.04180625295572488</v>
+        <v>0.05516354196624016</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>44.3989898989899</v>
+        <v>43.68787878787879</v>
       </c>
       <c r="B6">
-        <v>0.03480208572938091</v>
+        <v>0.04296524975839557</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>52.47373737373737</v>
+        <v>51.78484848484848</v>
       </c>
       <c r="B7">
-        <v>0.02987537705570119</v>
+        <v>0.03492127028347099</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>60.54848484848484</v>
+        <v>59.88181818181819</v>
       </c>
       <c r="B8">
-        <v>0.02621373526820083</v>
+        <v>0.02925286548600948</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>68.62323232323232</v>
+        <v>67.97878787878788</v>
       </c>
       <c r="B9">
-        <v>0.02338103360402072</v>
+        <v>0.02506208489084306</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.69797979797978</v>
+        <v>76.07575757575758</v>
       </c>
       <c r="B10">
-        <v>0.02112174936903392</v>
+        <v>0.02184900993129131</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.77272727272725</v>
+        <v>84.17272727272727</v>
       </c>
       <c r="B11">
-        <v>0.01927604335909764</v>
+        <v>0.01931428318245793</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.84747474747473</v>
+        <v>92.26969696969697</v>
       </c>
       <c r="B12">
-        <v>0.01773870091217781</v>
+        <v>0.01726822968450587</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.9222222222222</v>
+        <v>100.3666666666667</v>
       </c>
       <c r="B13">
-        <v>0.01643757540808223</v>
+        <v>0.01558512248656729</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.9969696969697</v>
+        <v>108.4636363636364</v>
       </c>
       <c r="B14">
-        <v>0.01532150915408134</v>
+        <v>0.01417848879016148</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>117.0717171717172</v>
+        <v>116.5606060606061</v>
       </c>
       <c r="B15">
-        <v>0.01435319723341663</v>
+        <v>0.01298699511530168</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>125.1464646464646</v>
+        <v>124.6575757575758</v>
       </c>
       <c r="B16">
-        <v>0.0135047825124472</v>
+        <v>0.01196599002919759</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>133.2212121212121</v>
+        <v>132.7545454545455</v>
       </c>
       <c r="B17">
-        <v>0.01275503402534345</v>
+        <v>0.0110822316650582</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>141.2959595959596</v>
+        <v>140.8515151515152</v>
       </c>
       <c r="B18">
-        <v>0.01208748145851442</v>
+        <v>0.01031048744007662</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>149.3707070707071</v>
+        <v>148.9484848484849</v>
       </c>
       <c r="B19">
-        <v>0.01148914749613198</v>
+        <v>0.009631275999786809</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.4454545454545</v>
+        <v>157.0454545454546</v>
       </c>
       <c r="B20">
-        <v>0.01094966553484734</v>
+        <v>0.009029328839544866</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.520202020202</v>
+        <v>165.1424242424243</v>
       </c>
       <c r="B21">
-        <v>0.01046065249826879</v>
+        <v>0.008492518339989152</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.5949494949495</v>
+        <v>173.2393939393939</v>
       </c>
       <c r="B22">
-        <v>0.01001525453838841</v>
+        <v>0.008011095705198019</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.6696969696969</v>
+        <v>181.3363636363637</v>
       </c>
       <c r="B23">
-        <v>0.009607812388484292</v>
+        <v>0.007577139428687919</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.7444444444444</v>
+        <v>189.4333333333334</v>
       </c>
       <c r="B24">
-        <v>0.009233611095551531</v>
+        <v>0.007184149648374311</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.8191919191919</v>
+        <v>197.5303030303031</v>
       </c>
       <c r="B25">
-        <v>0.008888690275485224</v>
+        <v>0.006826745424516108</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.8939393939393</v>
+        <v>205.6272727272728</v>
       </c>
       <c r="B26">
-        <v>0.00856969845168928</v>
+        <v>0.006500435816382649</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.9686868686868</v>
+        <v>213.7242424242424</v>
       </c>
       <c r="B27">
-        <v>0.008273779955781664</v>
+        <v>0.006201444662158525</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>222.0434343434343</v>
+        <v>221.8212121212121</v>
       </c>
       <c r="B28">
-        <v>0.007998486190224757</v>
+        <v>0.005926574970018011</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>230.1181818181818</v>
+        <v>229.9181818181818</v>
       </c>
       <c r="B29">
-        <v>0.007741705333417221</v>
+        <v>0.00567310289062023</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.1929292929293</v>
+        <v>238.0151515151516</v>
       </c>
       <c r="B30">
-        <v>0.007501606158254927</v>
+        <v>0.005438694034608454</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.2676767676767</v>
+        <v>246.1121212121213</v>
       </c>
       <c r="B31">
-        <v>0.007276592760105602</v>
+        <v>0.00522133684803717</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.3424242424242</v>
+        <v>254.2090909090909</v>
       </c>
       <c r="B32">
-        <v>0.007065267796277352</v>
+        <v>0.005019289137692525</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.4171717171717</v>
+        <v>262.3060606060606</v>
       </c>
       <c r="B33">
-        <v>0.006866402423782412</v>
+        <v>0.004831034826267896</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4919191919192</v>
+        <v>270.4030303030303</v>
       </c>
       <c r="B34">
-        <v>0.006678911551119365</v>
+        <v>0.0046552487335509</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5666666666667</v>
+        <v>278.5000000000001</v>
       </c>
       <c r="B35">
-        <v>0.006501833337750171</v>
+        <v>0.004490767704652825</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.6414141414141</v>
+        <v>286.5969696969697</v>
       </c>
       <c r="B36">
-        <v>0.006334312112962199</v>
+        <v>0.004336566794921568</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.7161616161616</v>
+        <v>294.6939393939394</v>
       </c>
       <c r="B37">
-        <v>0.006175584065620148</v>
+        <v>0.004191739511663775</v>
       </c>
     </row>
     <row r="38" spans="1:2">
@@ -3312,511 +3312,511 @@
         <v>302.7909090909091</v>
       </c>
       <c r="B38">
-        <v>0.006024965193333106</v>
+        <v>0.004055481331892936</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8656565656565</v>
+        <v>310.8878787878788</v>
       </c>
       <c r="B39">
-        <v>0.005881841104820782</v>
+        <v>0.003927075881962371</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.940404040404</v>
+        <v>318.9848484848485</v>
       </c>
       <c r="B40">
-        <v>0.005745658350741072</v>
+        <v>0.003805883292700867</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0151515151515</v>
+        <v>327.0818181818182</v>
       </c>
       <c r="B41">
-        <v>0.005615917021766245</v>
+        <v>0.003691330342352621</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.089898989899</v>
+        <v>335.1787878787879</v>
       </c>
       <c r="B42">
-        <v>0.005492164402560705</v>
+        <v>0.00358290207638999</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.1646464646465</v>
+        <v>343.2757575757576</v>
       </c>
       <c r="B43">
-        <v>0.005373989509709177</v>
+        <v>0.003480134653385886</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.2393939393939</v>
+        <v>351.3727272727273</v>
       </c>
       <c r="B44">
-        <v>0.005261018372958773</v>
+        <v>0.003382609213512734</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.3141414141414</v>
+        <v>359.469696969697</v>
       </c>
       <c r="B45">
-        <v>0.005152909944174143</v>
+        <v>0.003289946603801274</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.3888888888889</v>
+        <v>367.5666666666667</v>
       </c>
       <c r="B46">
-        <v>0.005049352538531013</v>
+        <v>0.003201802824248834</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.4636363636363</v>
+        <v>375.6636363636364</v>
       </c>
       <c r="B47">
-        <v>0.004950060728737752</v>
+        <v>0.003117865082885064</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.5383838383838</v>
+        <v>383.7606060606061</v>
       </c>
       <c r="B48">
-        <v>0.004854772626283929</v>
+        <v>0.003037848367260696</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.6131313131313</v>
+        <v>391.8575757575758</v>
       </c>
       <c r="B49">
-        <v>0.004763247494494139</v>
+        <v>0.002961492455503649</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.6878787878787</v>
+        <v>399.9545454545455</v>
       </c>
       <c r="B50">
-        <v>0.004675263647001852</v>
+        <v>0.002888559302845906</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>407.7626262626262</v>
+        <v>408.0515151515152</v>
       </c>
       <c r="B51">
-        <v>0.004590616592533375</v>
+        <v>0.002818830749954937</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>415.8373737373737</v>
+        <v>416.1484848484849</v>
       </c>
       <c r="B52">
-        <v>0.004509117392907075</v>
+        <v>0.002752106507966855</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>423.9121212121212</v>
+        <v>424.2454545454546</v>
       </c>
       <c r="B53">
-        <v>0.004430591206145848</v>
+        <v>0.002688202382178486</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>431.9868686868687</v>
+        <v>432.3424242424243</v>
       </c>
       <c r="B54">
-        <v>0.004354875990761184</v>
+        <v>0.002626948702199065</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.0616161616161</v>
+        <v>440.439393939394</v>
       </c>
       <c r="B55">
-        <v>0.004281821350746441</v>
+        <v>0.002568188931217557</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.1363636363636</v>
+        <v>448.5363636363637</v>
       </c>
       <c r="B56">
-        <v>0.004211287503737038</v>
+        <v>0.00251177843109041</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.2111111111111</v>
+        <v>456.6333333333334</v>
       </c>
       <c r="B57">
-        <v>0.00414314435725427</v>
+        <v>0.002457583363342884</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.2858585858585</v>
+        <v>464.7303030303031</v>
       </c>
       <c r="B58">
-        <v>0.00407727068002698</v>
+        <v>0.002405479709022215</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.360606060606</v>
+        <v>472.8272727272728</v>
       </c>
       <c r="B59">
-        <v>0.004013553357146009</v>
+        <v>0.002355352392737675</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.4353535353535</v>
+        <v>480.9242424242425</v>
       </c>
       <c r="B60">
-        <v>0.003951886719303136</v>
+        <v>0.002307094498248114</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>488.510101010101</v>
+        <v>489.0212121212122</v>
       </c>
       <c r="B61">
-        <v>0.003892171937642248</v>
+        <v>0.00226060656467445</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>496.5848484848485</v>
+        <v>497.1181818181819</v>
       </c>
       <c r="B62">
-        <v>0.003834316476841483</v>
+        <v>0.00221579595387411</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>504.6595959595959</v>
+        <v>505.2151515151515</v>
       </c>
       <c r="B63">
-        <v>0.003778233599980349</v>
+        <v>0.002172576280758743</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>512.7343434343434</v>
+        <v>513.3121212121213</v>
       </c>
       <c r="B64">
-        <v>0.003723841919549707</v>
+        <v>0.002130866899400167</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>520.8090909090909</v>
+        <v>521.4090909090909</v>
       </c>
       <c r="B65">
-        <v>0.003671064989655256</v>
+        <v>0.00209059243868117</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>528.8838383838383</v>
+        <v>529.5060606060606</v>
       </c>
       <c r="B66">
-        <v>0.003619830935063521</v>
+        <v>0.002051682382031121</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>536.9585858585858</v>
+        <v>537.6030303030303</v>
       </c>
       <c r="B67">
-        <v>0.003570072113257467</v>
+        <v>0.002014070686461129</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.0333333333333</v>
+        <v>545.7</v>
       </c>
       <c r="B68">
-        <v>0.003521724806118537</v>
+        <v>0.001977695436696093</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.1080808080808</v>
+        <v>553.7969696969697</v>
       </c>
       <c r="B69">
-        <v>0.003474728938243024</v>
+        <v>0.001942498530705191</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.1828282828283</v>
+        <v>561.8939393939394</v>
       </c>
       <c r="B70">
-        <v>0.003429027819241569</v>
+        <v>0.001908425393369704</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.2575757575758</v>
+        <v>569.9909090909091</v>
       </c>
       <c r="B71">
-        <v>0.003384567907668399</v>
+        <v>0.001875424715407219</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>577.3323232323232</v>
+        <v>578.0878787878788</v>
       </c>
       <c r="B72">
-        <v>0.003341298594487549</v>
+        <v>0.001843448215002397</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>585.4070707070706</v>
+        <v>586.1848484848484</v>
       </c>
       <c r="B73">
-        <v>0.00329917200421184</v>
+        <v>0.001812450419883519</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>593.4818181818181</v>
+        <v>594.2818181818182</v>
       </c>
       <c r="B74">
-        <v>0.003258142812051314</v>
+        <v>0.001782388467836827</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>601.5565656565656</v>
+        <v>602.3787878787879</v>
       </c>
       <c r="B75">
-        <v>0.003218168075584502</v>
+        <v>0.001753221923872184</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>609.631313131313</v>
+        <v>610.4757575757576</v>
       </c>
       <c r="B76">
-        <v>0.003179207079621927</v>
+        <v>0.001724912612448014</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>617.7060606060605</v>
+        <v>618.5727272727273</v>
       </c>
       <c r="B77">
-        <v>0.003141221193068869</v>
+        <v>0.001697424463334556</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>625.780808080808</v>
+        <v>626.6696969696969</v>
       </c>
       <c r="B78">
-        <v>0.003104173736716384</v>
+        <v>0.00167072336984511</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>633.8555555555555</v>
+        <v>634.7666666666667</v>
       </c>
       <c r="B79">
-        <v>0.003068029860997553</v>
+        <v>0.00164477705829798</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>641.930303030303</v>
+        <v>642.8636363636364</v>
       </c>
       <c r="B80">
-        <v>0.003032756432841862</v>
+        <v>0.001619554967689372</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.0050505050505</v>
+        <v>650.9606060606061</v>
       </c>
       <c r="B81">
-        <v>0.002998321930845916</v>
+        <v>0.001595028138661609</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>658.0797979797979</v>
+        <v>659.0575757575757</v>
       </c>
       <c r="B82">
-        <v>0.002964696348054624</v>
+        <v>0.001571169110943376</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>666.1545454545454</v>
+        <v>667.1545454545454</v>
       </c>
       <c r="B83">
-        <v>0.002931851101714743</v>
+        <v>0.001547951828520692</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>674.2292929292929</v>
+        <v>675.2515151515152</v>
       </c>
       <c r="B84">
-        <v>0.002899758949423204</v>
+        <v>0.001525351551870314</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>682.3040404040404</v>
+        <v>683.3484848484849</v>
       </c>
       <c r="B85">
-        <v>0.002868393911146696</v>
+        <v>0.001503344776652226</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>690.3787878787878</v>
+        <v>691.4454545454546</v>
       </c>
       <c r="B86">
-        <v>0.002837731196637552</v>
+        <v>0.001481909158315892</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>698.4535353535352</v>
+        <v>699.5424242424242</v>
       </c>
       <c r="B87">
-        <v>0.002807747137814382</v>
+        <v>0.001461023442126762</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>706.5282828282827</v>
+        <v>707.6393939393939</v>
       </c>
       <c r="B88">
-        <v>0.002778419125714995</v>
+        <v>0.001440667398165869</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>714.6030303030302</v>
+        <v>715.7363636363636</v>
       </c>
       <c r="B89">
-        <v>0.002749725551664224</v>
+        <v>0.001420821760896863</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>722.6777777777777</v>
+        <v>723.8333333333334</v>
       </c>
       <c r="B90">
-        <v>0.002721645752330935</v>
+        <v>0.001401468172932123</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>730.7525252525252</v>
+        <v>731.9303030303031</v>
       </c>
       <c r="B91">
-        <v>0.00269415995837694</v>
+        <v>0.001382589132662983</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>738.8272727272727</v>
+        <v>740.0272727272727</v>
       </c>
       <c r="B92">
-        <v>0.002667249246426297</v>
+        <v>0.001364167945449245</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>746.9020202020201</v>
+        <v>748.1242424242424</v>
       </c>
       <c r="B93">
-        <v>0.00264089549410671</v>
+        <v>0.001346188678090202</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>754.9767676767676</v>
+        <v>756.2212121212121</v>
       </c>
       <c r="B94">
-        <v>0.002615081337935753</v>
+        <v>0.001328636116323822</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>763.0515151515151</v>
+        <v>764.3181818181819</v>
       </c>
       <c r="B95">
-        <v>0.002589790133843706</v>
+        <v>0.001311495725122791</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>771.1262626262626</v>
+        <v>772.4151515151515</v>
       </c>
       <c r="B96">
-        <v>0.002565005920142038</v>
+        <v>0.00129475361157598</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>779.2010101010101</v>
+        <v>780.5121212121212</v>
       </c>
       <c r="B97">
-        <v>0.002540713382762229</v>
+        <v>0.001278396490161965</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>787.2757575757574</v>
+        <v>788.6090909090909</v>
       </c>
       <c r="B98">
-        <v>0.002516897822603894</v>
+        <v>0.001262411650237472</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>795.3505050505049</v>
+        <v>796.7060606060606</v>
       </c>
       <c r="B99">
-        <v>0.002493545124844073</v>
+        <v>0.001246786925578432</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>803.4252525252524</v>
+        <v>804.8030303030304</v>
       </c>
       <c r="B100">
-        <v>0.002470641730071381</v>
+        <v>0.001231510665824734</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>811.5</v>
+        <v>812.9</v>
       </c>
       <c r="B101">
-        <v>0.002448174607119392</v>
+        <v>0.001216571709691934</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
version 3.4.8: kernel-size vs nodes plot (remember zenodo after release)
</commit_message>
<xml_diff>
--- a/datasets/sgt_files/InVitroBioFilm_SGT_scaling.xlsx
+++ b/datasets/sgt_files/InVitroBioFilm_SGT_scaling.xlsx
@@ -440,25 +440,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="C2">
-        <v>1.3</v>
+        <v>1.408308678285174</v>
       </c>
       <c r="D2">
-        <v>0.223665</v>
+        <v>0.185419</v>
       </c>
       <c r="E2">
-        <v>0.08689313063566455</v>
+        <v>0.02764825308727077</v>
       </c>
       <c r="F2">
-        <v>1.05307844348342</v>
+        <v>1.021189299069938</v>
       </c>
       <c r="G2">
-        <v>-0.6504019707362143</v>
+        <v>-0.7318457654861891</v>
       </c>
       <c r="H2">
-        <v>-0.7360841467267152</v>
+        <v>-0.7956170590946079</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -466,25 +466,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39</v>
+        <v>38.1</v>
       </c>
       <c r="C3">
-        <v>3.0840089349921</v>
+        <v>1.27758452644912</v>
       </c>
       <c r="D3">
-        <v>0.047857</v>
+        <v>0.03847</v>
       </c>
       <c r="E3">
-        <v>0.005268825939218126</v>
+        <v>0.003421588649865569</v>
       </c>
       <c r="F3">
-        <v>1.591064607026499</v>
+        <v>1.580924975675619</v>
       </c>
       <c r="G3">
-        <v>-1.320054529380785</v>
+        <v>-1.414877813693185</v>
       </c>
       <c r="H3">
-        <v>-1.299983122420791</v>
+        <v>-1.347299254247706</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -492,25 +492,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>79.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="C4">
-        <v>2.478574859336174</v>
+        <v>2.394437999475729</v>
       </c>
       <c r="D4">
-        <v>0.01952</v>
+        <v>0.018984</v>
       </c>
       <c r="E4">
-        <v>0.001232376205187</v>
+        <v>0.00127096481287074</v>
       </c>
       <c r="F4">
-        <v>1.898176483497676</v>
+        <v>1.90848501887865</v>
       </c>
       <c r="G4">
-        <v>-1.709520186669327</v>
+        <v>-1.721612274790717</v>
       </c>
       <c r="H4">
-        <v>-1.621887446920606</v>
+        <v>-1.670146360893718</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -518,25 +518,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>130.9</v>
+        <v>137.5</v>
       </c>
       <c r="C5">
-        <v>4.787599723359411</v>
+        <v>4.185291706281256</v>
       </c>
       <c r="D5">
-        <v>0.012653</v>
+        <v>0.012357</v>
       </c>
       <c r="E5">
-        <v>0.001167132335636747</v>
+        <v>0.0007632111255886026</v>
       </c>
       <c r="F5">
-        <v>2.116939646550756</v>
+        <v>2.138302698166282</v>
       </c>
       <c r="G5">
-        <v>-1.897806491960256</v>
+        <v>-1.90808695332392</v>
       </c>
       <c r="H5">
-        <v>-1.851187625856062</v>
+        <v>-1.896657421548708</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -544,25 +544,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>214.1</v>
+        <v>211.1</v>
       </c>
       <c r="C6">
-        <v>4.670117771534247</v>
+        <v>5.722179072113467</v>
       </c>
       <c r="D6">
-        <v>0.007606</v>
+        <v>0.008705000000000001</v>
       </c>
       <c r="E6">
-        <v>0.000416579190817571</v>
+        <v>0.0005302289861727458</v>
       </c>
       <c r="F6">
-        <v>2.330616667294438</v>
+        <v>2.324488233307656</v>
       </c>
       <c r="G6">
-        <v>-2.118843678924436</v>
+        <v>-2.06023122454665</v>
       </c>
       <c r="H6">
-        <v>-2.075156681738808</v>
+        <v>-2.080164117701128</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -570,25 +570,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>288.1</v>
+        <v>287.4</v>
       </c>
       <c r="C7">
-        <v>5.685165882462103</v>
+        <v>3.679371927079101</v>
       </c>
       <c r="D7">
-        <v>0.00615</v>
+        <v>0.006292000000000001</v>
       </c>
       <c r="E7">
-        <v>0.0003635351121663185</v>
+        <v>0.0001936308056299124</v>
       </c>
       <c r="F7">
-        <v>2.459543258280413</v>
+        <v>2.458486763798207</v>
       </c>
       <c r="G7">
-        <v>-2.211124884224583</v>
+        <v>-2.201211286048751</v>
       </c>
       <c r="H7">
-        <v>-2.210293191789403</v>
+        <v>-2.212234676248701</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -596,25 +596,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>394</v>
+        <v>393.5</v>
       </c>
       <c r="C8">
-        <v>3.346640106136302</v>
+        <v>5.066776314603025</v>
       </c>
       <c r="D8">
-        <v>0.004235000000000001</v>
+        <v>0.004414</v>
       </c>
       <c r="E8">
-        <v>0.0001603347193287288</v>
+        <v>0.0002112144776182626</v>
       </c>
       <c r="F8">
-        <v>2.595496221825574</v>
+        <v>2.594944736695084</v>
       </c>
       <c r="G8">
-        <v>-2.373146585333274</v>
+        <v>-2.355167671174364</v>
       </c>
       <c r="H8">
-        <v>-2.352794508887963</v>
+        <v>-2.346729290725321</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -622,25 +622,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.2</v>
+        <v>515.3</v>
       </c>
       <c r="C9">
-        <v>3.805843460317889</v>
+        <v>7.935923946768195</v>
       </c>
       <c r="D9">
-        <v>0.003294</v>
+        <v>0.003261</v>
       </c>
       <c r="E9">
-        <v>0.0001124000790826136</v>
+        <v>0.0001578497879490358</v>
       </c>
       <c r="F9">
-        <v>2.711975854351756</v>
+        <v>2.712060142461075</v>
       </c>
       <c r="G9">
-        <v>-2.482276405166265</v>
+        <v>-2.486649201194043</v>
       </c>
       <c r="H9">
-        <v>-2.474884536330605</v>
+        <v>-2.462159639083738</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -648,25 +648,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>662.5</v>
+        <v>665.3</v>
       </c>
       <c r="C10">
-        <v>6.057593948462082</v>
+        <v>8.203048213926333</v>
       </c>
       <c r="D10">
-        <v>0.002638000000000001</v>
+        <v>0.002514</v>
       </c>
       <c r="E10">
-        <v>7.209253313161726E-05</v>
+        <v>0.0001025367142918954</v>
       </c>
       <c r="F10">
-        <v>2.821185882608845</v>
+        <v>2.823017523446049</v>
       </c>
       <c r="G10">
-        <v>-2.578725208789654</v>
+        <v>-2.599634726650061</v>
       </c>
       <c r="H10">
-        <v>-2.589354809439706</v>
+        <v>-2.571520564371608</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -674,25 +674,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="C11">
-        <v>9.599131905195039</v>
+        <v>7.651361534611556</v>
       </c>
       <c r="D11">
-        <v>0.00213</v>
+        <v>0.002173</v>
       </c>
       <c r="E11">
-        <v>6.881537295950343E-05</v>
+        <v>6.824872811187685E-05</v>
       </c>
       <c r="F11">
-        <v>2.910037123553051</v>
+        <v>2.904769625906595</v>
       </c>
       <c r="G11">
-        <v>-2.671620396561262</v>
+        <v>-2.662940273679475</v>
       </c>
       <c r="H11">
-        <v>-2.68248568743035</v>
+        <v>-2.652096416919216</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -718,7 +718,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.457595894667791</v>
+        <v>-2.445819704215646</v>
       </c>
     </row>
   </sheetData>
@@ -741,802 +741,802 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="B2">
-        <v>0.2234229411226657</v>
+        <v>0.184891647846076</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>19.3969696969697</v>
+        <v>18.50606060606061</v>
       </c>
       <c r="B3">
-        <v>0.1156212373834673</v>
+        <v>0.09699386650165555</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>27.4939393939394</v>
+        <v>26.51212121212121</v>
       </c>
       <c r="B4">
-        <v>0.07556595810281702</v>
+        <v>0.06441915600835781</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>35.59090909090909</v>
+        <v>34.51818181818182</v>
       </c>
       <c r="B5">
-        <v>0.05516354196624016</v>
+        <v>0.04770430921186292</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>43.68787878787879</v>
+        <v>42.52424242424242</v>
       </c>
       <c r="B6">
-        <v>0.04296524975839557</v>
+        <v>0.03762158624308524</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>51.78484848484848</v>
+        <v>50.53030303030303</v>
       </c>
       <c r="B7">
-        <v>0.03492127028347099</v>
+        <v>0.03091421103869369</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>59.88181818181819</v>
+        <v>58.53636363636363</v>
       </c>
       <c r="B8">
-        <v>0.02925286548600948</v>
+        <v>0.02614858339296097</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>67.97878787878788</v>
+        <v>66.54242424242423</v>
       </c>
       <c r="B9">
-        <v>0.02506208489084306</v>
+        <v>0.02259818839391243</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.07575757575758</v>
+        <v>74.54848484848485</v>
       </c>
       <c r="B10">
-        <v>0.02184900993129131</v>
+        <v>0.01985673358482553</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.17272727272727</v>
+        <v>82.55454545454545</v>
       </c>
       <c r="B11">
-        <v>0.01931428318245793</v>
+        <v>0.01767978487064297</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.26969696969697</v>
+        <v>90.56060606060606</v>
       </c>
       <c r="B12">
-        <v>0.01726822968450587</v>
+        <v>0.01591174092637995</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.3666666666667</v>
+        <v>98.56666666666666</v>
       </c>
       <c r="B13">
-        <v>0.01558512248656729</v>
+        <v>0.01444898696256113</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.4636363636364</v>
+        <v>106.5727272727273</v>
       </c>
       <c r="B14">
-        <v>0.01417848879016148</v>
+        <v>0.01321994121343388</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>116.5606060606061</v>
+        <v>114.5787878787879</v>
       </c>
       <c r="B15">
-        <v>0.01298699511530168</v>
+        <v>0.01217361410153211</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>124.6575757575758</v>
+        <v>122.5848484848485</v>
       </c>
       <c r="B16">
-        <v>0.01196599002919759</v>
+        <v>0.01127273135110265</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>132.7545454545455</v>
+        <v>130.5909090909091</v>
       </c>
       <c r="B17">
-        <v>0.0110822316650582</v>
+        <v>0.01048943309212318</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>140.8515151515152</v>
+        <v>138.5969696969697</v>
       </c>
       <c r="B18">
-        <v>0.01031048744007662</v>
+        <v>0.009802491403436467</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>148.9484848484849</v>
+        <v>146.6030303030303</v>
       </c>
       <c r="B19">
-        <v>0.009631275999786809</v>
+        <v>0.009195456799216902</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.0454545454546</v>
+        <v>154.6090909090909</v>
       </c>
       <c r="B20">
-        <v>0.009029328839544866</v>
+        <v>0.008655391614442896</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.1424242424243</v>
+        <v>162.6151515151515</v>
       </c>
       <c r="B21">
-        <v>0.008492518339989152</v>
+        <v>0.008171984784864205</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.2393939393939</v>
+        <v>170.6212121212121</v>
       </c>
       <c r="B22">
-        <v>0.008011095705198019</v>
+        <v>0.007736920717535016</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.3363636363637</v>
+        <v>178.6272727272727</v>
       </c>
       <c r="B23">
-        <v>0.007577139428687919</v>
+        <v>0.007343421227736977</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.4333333333334</v>
+        <v>186.6333333333333</v>
       </c>
       <c r="B24">
-        <v>0.007184149648374311</v>
+        <v>0.006985907714317893</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.5303030303031</v>
+        <v>194.6393939393939</v>
       </c>
       <c r="B25">
-        <v>0.006826745424516108</v>
+        <v>0.006659748375801701</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.6272727272728</v>
+        <v>202.6454545454545</v>
       </c>
       <c r="B26">
-        <v>0.006500435816382649</v>
+        <v>0.006361066553561816</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.7242424242424</v>
+        <v>210.6515151515152</v>
       </c>
       <c r="B27">
-        <v>0.006201444662158525</v>
+        <v>0.006086593664304345</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>221.8212121212121</v>
+        <v>218.6575757575758</v>
       </c>
       <c r="B28">
-        <v>0.005926574970018011</v>
+        <v>0.005833555098793225</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>229.9181818181818</v>
+        <v>226.6636363636364</v>
       </c>
       <c r="B29">
-        <v>0.00567310289062023</v>
+        <v>0.005599580796224393</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.0151515151516</v>
+        <v>234.669696969697</v>
       </c>
       <c r="B30">
-        <v>0.005438694034608454</v>
+        <v>0.005382634499791695</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.1121212121213</v>
+        <v>242.6757575757576</v>
       </c>
       <c r="B31">
-        <v>0.00522133684803717</v>
+        <v>0.005180957304561919</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.2090909090909</v>
+        <v>250.6818181818182</v>
       </c>
       <c r="B32">
-        <v>0.005019289137692525</v>
+        <v>0.004993022246858652</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.3060606060606</v>
+        <v>258.6878787878788</v>
       </c>
       <c r="B33">
-        <v>0.004831034826267896</v>
+        <v>0.004817497501294103</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4030303030303</v>
+        <v>266.6939393939394</v>
       </c>
       <c r="B34">
-        <v>0.0046552487335509</v>
+        <v>0.004653216344908505</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5000000000001</v>
+        <v>274.7</v>
       </c>
       <c r="B35">
-        <v>0.004490767704652825</v>
+        <v>0.004499152483511465</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.5969696969697</v>
+        <v>282.7060606060606</v>
       </c>
       <c r="B36">
-        <v>0.004336566794921568</v>
+        <v>0.00435439965844809</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.6939393939394</v>
+        <v>290.7121212121212</v>
       </c>
       <c r="B37">
-        <v>0.004191739511663775</v>
+        <v>0.004218154693983959</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38">
-        <v>302.7909090909091</v>
+        <v>298.7181818181818</v>
       </c>
       <c r="B38">
-        <v>0.004055481331892936</v>
+        <v>0.004089703328325833</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8878787878788</v>
+        <v>306.7242424242424</v>
       </c>
       <c r="B39">
-        <v>0.003927075881962371</v>
+        <v>0.003968408310592312</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.9848484848485</v>
+        <v>314.730303030303</v>
       </c>
       <c r="B40">
-        <v>0.003805883292700867</v>
+        <v>0.003853699353024394</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0818181818182</v>
+        <v>322.7363636363636</v>
       </c>
       <c r="B41">
-        <v>0.003691330342352621</v>
+        <v>0.003745064610494677</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.1787878787879</v>
+        <v>330.7424242424242</v>
       </c>
       <c r="B42">
-        <v>0.00358290207638999</v>
+        <v>0.003642043423865678</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.2757575757576</v>
+        <v>338.7484848484848</v>
       </c>
       <c r="B43">
-        <v>0.003480134653385886</v>
+        <v>0.003544220114334572</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.3727272727273</v>
+        <v>346.7545454545455</v>
       </c>
       <c r="B44">
-        <v>0.003382609213512734</v>
+        <v>0.003451218655832776</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.469696969697</v>
+        <v>354.7606060606061</v>
       </c>
       <c r="B45">
-        <v>0.003289946603801274</v>
+        <v>0.003362698084258411</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.5666666666667</v>
+        <v>362.7666666666667</v>
       </c>
       <c r="B46">
-        <v>0.003201802824248834</v>
+        <v>0.003278348527644262</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.6636363636364</v>
+        <v>370.7727272727273</v>
       </c>
       <c r="B47">
-        <v>0.003117865082885064</v>
+        <v>0.003197887761699077</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.7606060606061</v>
+        <v>378.7787878787879</v>
       </c>
       <c r="B48">
-        <v>0.003037848367260696</v>
+        <v>0.003121058211573426</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.8575757575758</v>
+        <v>386.7848484848485</v>
       </c>
       <c r="B49">
-        <v>0.002961492455503649</v>
+        <v>0.003047624334014674</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.9545454545455</v>
+        <v>394.7909090909091</v>
       </c>
       <c r="B50">
-        <v>0.002888559302845906</v>
+        <v>0.002977370324925316</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>408.0515151515152</v>
+        <v>402.7969696969697</v>
       </c>
       <c r="B51">
-        <v>0.002818830749954937</v>
+        <v>0.002910098106220766</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>416.1484848484849</v>
+        <v>410.8030303030303</v>
       </c>
       <c r="B52">
-        <v>0.002752106507966855</v>
+        <v>0.002845625553184896</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>424.2454545454546</v>
+        <v>418.8090909090909</v>
       </c>
       <c r="B53">
-        <v>0.002688202382178486</v>
+        <v>0.002783784929549944</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>432.3424242424243</v>
+        <v>426.8151515151515</v>
       </c>
       <c r="B54">
-        <v>0.002626948702199065</v>
+        <v>0.002724421502523833</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.439393939394</v>
+        <v>434.8212121212121</v>
       </c>
       <c r="B55">
-        <v>0.002568188931217557</v>
+        <v>0.002667392314144691</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.5363636363637</v>
+        <v>442.8272727272727</v>
       </c>
       <c r="B56">
-        <v>0.00251177843109041</v>
+        <v>0.00261256508881331</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.6333333333334</v>
+        <v>450.8333333333333</v>
       </c>
       <c r="B57">
-        <v>0.002457583363342884</v>
+        <v>0.00255981725976266</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.7303030303031</v>
+        <v>458.8393939393939</v>
       </c>
       <c r="B58">
-        <v>0.002405479709022215</v>
+        <v>0.002509035099668747</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.8272727272728</v>
+        <v>466.8454545454545</v>
       </c>
       <c r="B59">
-        <v>0.002355352392737675</v>
+        <v>0.002460112942669601</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.9242424242425</v>
+        <v>474.8515151515151</v>
       </c>
       <c r="B60">
-        <v>0.002307094498248114</v>
+        <v>0.002412952486804241</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>489.0212121212122</v>
+        <v>482.8575757575758</v>
       </c>
       <c r="B61">
-        <v>0.00226060656467445</v>
+        <v>0.002367462167364444</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>497.1181818181819</v>
+        <v>490.8636363636364</v>
       </c>
       <c r="B62">
-        <v>0.00221579595387411</v>
+        <v>0.002323556592912663</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>505.2151515151515</v>
+        <v>498.869696969697</v>
       </c>
       <c r="B63">
-        <v>0.002172576280758743</v>
+        <v>0.002281156036795257</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>513.3121212121213</v>
+        <v>506.8757575757576</v>
       </c>
       <c r="B64">
-        <v>0.002130866899400167</v>
+        <v>0.002240185977900962</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>521.4090909090909</v>
+        <v>514.8818181818182</v>
       </c>
       <c r="B65">
-        <v>0.00209059243868117</v>
+        <v>0.002200576685204554</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>529.5060606060606</v>
+        <v>522.8878787878788</v>
       </c>
       <c r="B66">
-        <v>0.002051682382031121</v>
+        <v>0.002162262841315321</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>537.6030303030303</v>
+        <v>530.8939393939394</v>
       </c>
       <c r="B67">
-        <v>0.002014070686461129</v>
+        <v>0.002125183200835971</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.7</v>
+        <v>538.9</v>
       </c>
       <c r="B68">
-        <v>0.001977695436696093</v>
+        <v>0.002089280279844253</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.7969696969697</v>
+        <v>546.9060606060606</v>
       </c>
       <c r="B69">
-        <v>0.001942498530705191</v>
+        <v>0.002054500073248407</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.8939393939394</v>
+        <v>554.9121212121212</v>
       </c>
       <c r="B70">
-        <v>0.001908425393369704</v>
+        <v>0.002020791797148658</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.9909090909091</v>
+        <v>562.9181818181818</v>
       </c>
       <c r="B71">
-        <v>0.001875424715407219</v>
+        <v>0.001988107653668595</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>578.0878787878788</v>
+        <v>570.9242424242424</v>
       </c>
       <c r="B72">
-        <v>0.001843448215002397</v>
+        <v>0.001956402616009377</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>586.1848484848484</v>
+        <v>578.930303030303</v>
       </c>
       <c r="B73">
-        <v>0.001812450419883519</v>
+        <v>0.001925634231732409</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>594.2818181818182</v>
+        <v>586.9363636363636</v>
       </c>
       <c r="B74">
-        <v>0.001782388467836827</v>
+        <v>0.00189576244249727</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>602.3787878787879</v>
+        <v>594.9424242424242</v>
       </c>
       <c r="B75">
-        <v>0.001753221923872184</v>
+        <v>0.001866749418675721</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>610.4757575757576</v>
+        <v>602.9484848484848</v>
       </c>
       <c r="B76">
-        <v>0.001724912612448014</v>
+        <v>0.001838559407433083</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>618.5727272727273</v>
+        <v>610.9545454545455</v>
       </c>
       <c r="B77">
-        <v>0.001697424463334556</v>
+        <v>0.00181115859301838</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>626.6696969696969</v>
+        <v>618.9606060606061</v>
       </c>
       <c r="B78">
-        <v>0.00167072336984511</v>
+        <v>0.001784514968137032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>634.7666666666667</v>
+        <v>626.9666666666667</v>
       </c>
       <c r="B79">
-        <v>0.00164477705829798</v>
+        <v>0.001758598215396764</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>642.8636363636364</v>
+        <v>634.9727272727273</v>
       </c>
       <c r="B80">
-        <v>0.001619554967689372</v>
+        <v>0.001733379597920934</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.9606060606061</v>
+        <v>642.9787878787879</v>
       </c>
       <c r="B81">
-        <v>0.001595028138661609</v>
+        <v>0.001708831858315155</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>659.0575757575757</v>
+        <v>650.9848484848485</v>
       </c>
       <c r="B82">
-        <v>0.001571169110943376</v>
+        <v>0.001684929125254508</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>667.1545454545454</v>
+        <v>658.9909090909091</v>
       </c>
       <c r="B83">
-        <v>0.001547951828520692</v>
+        <v>0.001661646827031027</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>675.2515151515152</v>
+        <v>666.9969696969697</v>
       </c>
       <c r="B84">
-        <v>0.001525351551870314</v>
+        <v>0.001638961611465592</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>683.3484848484849</v>
+        <v>675.0030303030303</v>
       </c>
       <c r="B85">
-        <v>0.001503344776652226</v>
+        <v>0.001616851271645816</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>691.4454545454546</v>
+        <v>683.0090909090909</v>
       </c>
       <c r="B86">
-        <v>0.001481909158315892</v>
+        <v>0.001595294677002861</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>699.5424242424242</v>
+        <v>691.0151515151515</v>
       </c>
       <c r="B87">
-        <v>0.001461023442126762</v>
+        <v>0.001574271709285973</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>707.6393939393939</v>
+        <v>699.0212121212121</v>
       </c>
       <c r="B88">
-        <v>0.001440667398165869</v>
+        <v>0.001553763203034644</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>715.7363636363636</v>
+        <v>707.0272727272727</v>
       </c>
       <c r="B89">
-        <v>0.001420821760896863</v>
+        <v>0.001533750890185145</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>723.8333333333334</v>
+        <v>715.0333333333333</v>
       </c>
       <c r="B90">
-        <v>0.001401468172932123</v>
+        <v>0.001514217348481232</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>731.9303030303031</v>
+        <v>723.0393939393939</v>
       </c>
       <c r="B91">
-        <v>0.001382589132662983</v>
+        <v>0.001495145953388581</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>740.0272727272727</v>
+        <v>731.0454545454545</v>
       </c>
       <c r="B92">
-        <v>0.001364167945449245</v>
+        <v>0.001476520833239256</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>748.1242424242424</v>
+        <v>739.0515151515151</v>
       </c>
       <c r="B93">
-        <v>0.001346188678090202</v>
+        <v>0.00145832682735662</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>756.2212121212121</v>
+        <v>747.0575757575757</v>
       </c>
       <c r="B94">
-        <v>0.001328636116323822</v>
+        <v>0.001440549446932866</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>764.3181818181819</v>
+        <v>755.0636363636363</v>
       </c>
       <c r="B95">
-        <v>0.001311495725122791</v>
+        <v>0.001423174838450966</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>772.4151515151515</v>
+        <v>763.0696969696969</v>
       </c>
       <c r="B96">
-        <v>0.00129475361157598</v>
+        <v>0.001406189749460629</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>780.5121212121212</v>
+        <v>771.0757575757575</v>
       </c>
       <c r="B97">
-        <v>0.001278396490161965</v>
+        <v>0.001389581496533911</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>788.6090909090909</v>
+        <v>779.0818181818181</v>
       </c>
       <c r="B98">
-        <v>0.001262411650237472</v>
+        <v>0.00137333793524071</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>796.7060606060606</v>
+        <v>787.0878787878788</v>
       </c>
       <c r="B99">
-        <v>0.001246786925578432</v>
+        <v>0.001357447431997586</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>804.8030303030304</v>
+        <v>795.0939393939394</v>
       </c>
       <c r="B100">
-        <v>0.001231510665824734</v>
+        <v>0.00134189883765535</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="B101">
-        <v>0.001216571709691934</v>
+        <v>0.00132668146270177</v>
       </c>
     </row>
   </sheetData>
@@ -1580,25 +1580,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="C2">
-        <v>1.3</v>
+        <v>1.408308678285174</v>
       </c>
       <c r="D2">
-        <v>0.223665</v>
+        <v>0.185419</v>
       </c>
       <c r="E2">
-        <v>0.08689313063566455</v>
+        <v>0.02764825308727077</v>
       </c>
       <c r="F2">
-        <v>1.05307844348342</v>
+        <v>1.021189299069938</v>
       </c>
       <c r="G2">
-        <v>-0.6504019707362143</v>
+        <v>-0.7318457654861891</v>
       </c>
       <c r="H2">
-        <v>-0.7360841467267152</v>
+        <v>-0.7956170590946079</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -1606,25 +1606,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39</v>
+        <v>38.1</v>
       </c>
       <c r="C3">
-        <v>3.0840089349921</v>
+        <v>1.27758452644912</v>
       </c>
       <c r="D3">
-        <v>0.047857</v>
+        <v>0.03847</v>
       </c>
       <c r="E3">
-        <v>0.005268825939218126</v>
+        <v>0.003421588649865569</v>
       </c>
       <c r="F3">
-        <v>1.591064607026499</v>
+        <v>1.580924975675619</v>
       </c>
       <c r="G3">
-        <v>-1.320054529380785</v>
+        <v>-1.414877813693185</v>
       </c>
       <c r="H3">
-        <v>-1.299983122420791</v>
+        <v>-1.347299254247706</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -1632,25 +1632,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>79.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="C4">
-        <v>2.478574859336174</v>
+        <v>2.394437999475729</v>
       </c>
       <c r="D4">
-        <v>0.01952</v>
+        <v>0.018984</v>
       </c>
       <c r="E4">
-        <v>0.001232376205187</v>
+        <v>0.00127096481287074</v>
       </c>
       <c r="F4">
-        <v>1.898176483497676</v>
+        <v>1.90848501887865</v>
       </c>
       <c r="G4">
-        <v>-1.709520186669327</v>
+        <v>-1.721612274790717</v>
       </c>
       <c r="H4">
-        <v>-1.621887446920606</v>
+        <v>-1.670146360893718</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -1658,25 +1658,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>130.9</v>
+        <v>137.5</v>
       </c>
       <c r="C5">
-        <v>4.787599723359411</v>
+        <v>4.185291706281256</v>
       </c>
       <c r="D5">
-        <v>0.012653</v>
+        <v>0.012357</v>
       </c>
       <c r="E5">
-        <v>0.001167132335636747</v>
+        <v>0.0007632111255886026</v>
       </c>
       <c r="F5">
-        <v>2.116939646550756</v>
+        <v>2.138302698166282</v>
       </c>
       <c r="G5">
-        <v>-1.897806491960256</v>
+        <v>-1.90808695332392</v>
       </c>
       <c r="H5">
-        <v>-1.851187625856062</v>
+        <v>-1.896657421548708</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -1684,25 +1684,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>214.1</v>
+        <v>211.1</v>
       </c>
       <c r="C6">
-        <v>4.670117771534247</v>
+        <v>5.722179072113467</v>
       </c>
       <c r="D6">
-        <v>0.007606</v>
+        <v>0.008705000000000001</v>
       </c>
       <c r="E6">
-        <v>0.000416579190817571</v>
+        <v>0.0005302289861727458</v>
       </c>
       <c r="F6">
-        <v>2.330616667294438</v>
+        <v>2.324488233307656</v>
       </c>
       <c r="G6">
-        <v>-2.118843678924436</v>
+        <v>-2.06023122454665</v>
       </c>
       <c r="H6">
-        <v>-2.075156681738808</v>
+        <v>-2.080164117701128</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -1710,25 +1710,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>288.1</v>
+        <v>287.4</v>
       </c>
       <c r="C7">
-        <v>5.685165882462103</v>
+        <v>3.679371927079101</v>
       </c>
       <c r="D7">
-        <v>0.00615</v>
+        <v>0.006292000000000001</v>
       </c>
       <c r="E7">
-        <v>0.0003635351121663185</v>
+        <v>0.0001936308056299124</v>
       </c>
       <c r="F7">
-        <v>2.459543258280413</v>
+        <v>2.458486763798207</v>
       </c>
       <c r="G7">
-        <v>-2.211124884224583</v>
+        <v>-2.201211286048751</v>
       </c>
       <c r="H7">
-        <v>-2.210293191789403</v>
+        <v>-2.212234676248701</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -1736,25 +1736,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>394</v>
+        <v>393.5</v>
       </c>
       <c r="C8">
-        <v>3.346640106136302</v>
+        <v>5.066776314603025</v>
       </c>
       <c r="D8">
-        <v>0.004235000000000001</v>
+        <v>0.004414</v>
       </c>
       <c r="E8">
-        <v>0.0001603347193287288</v>
+        <v>0.0002112144776182626</v>
       </c>
       <c r="F8">
-        <v>2.595496221825574</v>
+        <v>2.594944736695084</v>
       </c>
       <c r="G8">
-        <v>-2.373146585333274</v>
+        <v>-2.355167671174364</v>
       </c>
       <c r="H8">
-        <v>-2.352794508887963</v>
+        <v>-2.346729290725321</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -1762,25 +1762,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.2</v>
+        <v>515.3</v>
       </c>
       <c r="C9">
-        <v>3.805843460317889</v>
+        <v>7.935923946768195</v>
       </c>
       <c r="D9">
-        <v>0.003294</v>
+        <v>0.003261</v>
       </c>
       <c r="E9">
-        <v>0.0001124000790826136</v>
+        <v>0.0001578497879490358</v>
       </c>
       <c r="F9">
-        <v>2.711975854351756</v>
+        <v>2.712060142461075</v>
       </c>
       <c r="G9">
-        <v>-2.482276405166265</v>
+        <v>-2.486649201194043</v>
       </c>
       <c r="H9">
-        <v>-2.474884536330605</v>
+        <v>-2.462159639083738</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -1788,25 +1788,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>662.5</v>
+        <v>665.3</v>
       </c>
       <c r="C10">
-        <v>6.057593948462082</v>
+        <v>8.203048213926333</v>
       </c>
       <c r="D10">
-        <v>0.002638000000000001</v>
+        <v>0.002514</v>
       </c>
       <c r="E10">
-        <v>7.209253313161726E-05</v>
+        <v>0.0001025367142918954</v>
       </c>
       <c r="F10">
-        <v>2.821185882608845</v>
+        <v>2.823017523446049</v>
       </c>
       <c r="G10">
-        <v>-2.578725208789654</v>
+        <v>-2.599634726650061</v>
       </c>
       <c r="H10">
-        <v>-2.589354809439706</v>
+        <v>-2.571520564371608</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -1814,25 +1814,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="C11">
-        <v>9.599131905195039</v>
+        <v>7.651361534611556</v>
       </c>
       <c r="D11">
-        <v>0.00213</v>
+        <v>0.002173</v>
       </c>
       <c r="E11">
-        <v>6.881537295950343E-05</v>
+        <v>6.824872811187685E-05</v>
       </c>
       <c r="F11">
-        <v>2.910037123553051</v>
+        <v>2.904769625906595</v>
       </c>
       <c r="G11">
-        <v>-2.671620396561262</v>
+        <v>-2.662940273679475</v>
       </c>
       <c r="H11">
-        <v>-2.68248568743035</v>
+        <v>-2.652096416919216</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -1858,7 +1858,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.457595894667791</v>
+        <v>-2.445819704215646</v>
       </c>
     </row>
   </sheetData>
@@ -1881,802 +1881,802 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="B2">
-        <v>0.2234229411226657</v>
+        <v>0.184891647846076</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>19.3969696969697</v>
+        <v>18.50606060606061</v>
       </c>
       <c r="B3">
-        <v>0.1156212373834673</v>
+        <v>0.09699386650165555</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>27.4939393939394</v>
+        <v>26.51212121212121</v>
       </c>
       <c r="B4">
-        <v>0.07556595810281702</v>
+        <v>0.06441915600835781</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>35.59090909090909</v>
+        <v>34.51818181818182</v>
       </c>
       <c r="B5">
-        <v>0.05516354196624016</v>
+        <v>0.04770430921186292</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>43.68787878787879</v>
+        <v>42.52424242424242</v>
       </c>
       <c r="B6">
-        <v>0.04296524975839557</v>
+        <v>0.03762158624308524</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>51.78484848484848</v>
+        <v>50.53030303030303</v>
       </c>
       <c r="B7">
-        <v>0.03492127028347099</v>
+        <v>0.03091421103869369</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>59.88181818181819</v>
+        <v>58.53636363636363</v>
       </c>
       <c r="B8">
-        <v>0.02925286548600948</v>
+        <v>0.02614858339296097</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>67.97878787878788</v>
+        <v>66.54242424242423</v>
       </c>
       <c r="B9">
-        <v>0.02506208489084306</v>
+        <v>0.02259818839391243</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.07575757575758</v>
+        <v>74.54848484848485</v>
       </c>
       <c r="B10">
-        <v>0.02184900993129131</v>
+        <v>0.01985673358482553</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.17272727272727</v>
+        <v>82.55454545454545</v>
       </c>
       <c r="B11">
-        <v>0.01931428318245793</v>
+        <v>0.01767978487064297</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.26969696969697</v>
+        <v>90.56060606060606</v>
       </c>
       <c r="B12">
-        <v>0.01726822968450587</v>
+        <v>0.01591174092637995</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.3666666666667</v>
+        <v>98.56666666666666</v>
       </c>
       <c r="B13">
-        <v>0.01558512248656729</v>
+        <v>0.01444898696256113</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.4636363636364</v>
+        <v>106.5727272727273</v>
       </c>
       <c r="B14">
-        <v>0.01417848879016148</v>
+        <v>0.01321994121343388</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>116.5606060606061</v>
+        <v>114.5787878787879</v>
       </c>
       <c r="B15">
-        <v>0.01298699511530168</v>
+        <v>0.01217361410153211</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>124.6575757575758</v>
+        <v>122.5848484848485</v>
       </c>
       <c r="B16">
-        <v>0.01196599002919759</v>
+        <v>0.01127273135110265</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>132.7545454545455</v>
+        <v>130.5909090909091</v>
       </c>
       <c r="B17">
-        <v>0.0110822316650582</v>
+        <v>0.01048943309212318</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>140.8515151515152</v>
+        <v>138.5969696969697</v>
       </c>
       <c r="B18">
-        <v>0.01031048744007662</v>
+        <v>0.009802491403436467</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>148.9484848484849</v>
+        <v>146.6030303030303</v>
       </c>
       <c r="B19">
-        <v>0.009631275999786809</v>
+        <v>0.009195456799216902</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.0454545454546</v>
+        <v>154.6090909090909</v>
       </c>
       <c r="B20">
-        <v>0.009029328839544866</v>
+        <v>0.008655391614442896</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.1424242424243</v>
+        <v>162.6151515151515</v>
       </c>
       <c r="B21">
-        <v>0.008492518339989152</v>
+        <v>0.008171984784864205</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.2393939393939</v>
+        <v>170.6212121212121</v>
       </c>
       <c r="B22">
-        <v>0.008011095705198019</v>
+        <v>0.007736920717535016</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.3363636363637</v>
+        <v>178.6272727272727</v>
       </c>
       <c r="B23">
-        <v>0.007577139428687919</v>
+        <v>0.007343421227736977</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.4333333333334</v>
+        <v>186.6333333333333</v>
       </c>
       <c r="B24">
-        <v>0.007184149648374311</v>
+        <v>0.006985907714317893</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.5303030303031</v>
+        <v>194.6393939393939</v>
       </c>
       <c r="B25">
-        <v>0.006826745424516108</v>
+        <v>0.006659748375801701</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.6272727272728</v>
+        <v>202.6454545454545</v>
       </c>
       <c r="B26">
-        <v>0.006500435816382649</v>
+        <v>0.006361066553561816</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.7242424242424</v>
+        <v>210.6515151515152</v>
       </c>
       <c r="B27">
-        <v>0.006201444662158525</v>
+        <v>0.006086593664304345</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>221.8212121212121</v>
+        <v>218.6575757575758</v>
       </c>
       <c r="B28">
-        <v>0.005926574970018011</v>
+        <v>0.005833555098793225</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>229.9181818181818</v>
+        <v>226.6636363636364</v>
       </c>
       <c r="B29">
-        <v>0.00567310289062023</v>
+        <v>0.005599580796224393</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.0151515151516</v>
+        <v>234.669696969697</v>
       </c>
       <c r="B30">
-        <v>0.005438694034608454</v>
+        <v>0.005382634499791695</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.1121212121213</v>
+        <v>242.6757575757576</v>
       </c>
       <c r="B31">
-        <v>0.00522133684803717</v>
+        <v>0.005180957304561919</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.2090909090909</v>
+        <v>250.6818181818182</v>
       </c>
       <c r="B32">
-        <v>0.005019289137692525</v>
+        <v>0.004993022246858652</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.3060606060606</v>
+        <v>258.6878787878788</v>
       </c>
       <c r="B33">
-        <v>0.004831034826267896</v>
+        <v>0.004817497501294103</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4030303030303</v>
+        <v>266.6939393939394</v>
       </c>
       <c r="B34">
-        <v>0.0046552487335509</v>
+        <v>0.004653216344908505</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5000000000001</v>
+        <v>274.7</v>
       </c>
       <c r="B35">
-        <v>0.004490767704652825</v>
+        <v>0.004499152483511465</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.5969696969697</v>
+        <v>282.7060606060606</v>
       </c>
       <c r="B36">
-        <v>0.004336566794921568</v>
+        <v>0.00435439965844809</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.6939393939394</v>
+        <v>290.7121212121212</v>
       </c>
       <c r="B37">
-        <v>0.004191739511663775</v>
+        <v>0.004218154693983959</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38">
-        <v>302.7909090909091</v>
+        <v>298.7181818181818</v>
       </c>
       <c r="B38">
-        <v>0.004055481331892936</v>
+        <v>0.004089703328325833</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8878787878788</v>
+        <v>306.7242424242424</v>
       </c>
       <c r="B39">
-        <v>0.003927075881962371</v>
+        <v>0.003968408310592312</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.9848484848485</v>
+        <v>314.730303030303</v>
       </c>
       <c r="B40">
-        <v>0.003805883292700867</v>
+        <v>0.003853699353024394</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0818181818182</v>
+        <v>322.7363636363636</v>
       </c>
       <c r="B41">
-        <v>0.003691330342352621</v>
+        <v>0.003745064610494677</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.1787878787879</v>
+        <v>330.7424242424242</v>
       </c>
       <c r="B42">
-        <v>0.00358290207638999</v>
+        <v>0.003642043423865678</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.2757575757576</v>
+        <v>338.7484848484848</v>
       </c>
       <c r="B43">
-        <v>0.003480134653385886</v>
+        <v>0.003544220114334572</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.3727272727273</v>
+        <v>346.7545454545455</v>
       </c>
       <c r="B44">
-        <v>0.003382609213512734</v>
+        <v>0.003451218655832776</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.469696969697</v>
+        <v>354.7606060606061</v>
       </c>
       <c r="B45">
-        <v>0.003289946603801274</v>
+        <v>0.003362698084258411</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.5666666666667</v>
+        <v>362.7666666666667</v>
       </c>
       <c r="B46">
-        <v>0.003201802824248834</v>
+        <v>0.003278348527644262</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.6636363636364</v>
+        <v>370.7727272727273</v>
       </c>
       <c r="B47">
-        <v>0.003117865082885064</v>
+        <v>0.003197887761699077</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.7606060606061</v>
+        <v>378.7787878787879</v>
       </c>
       <c r="B48">
-        <v>0.003037848367260696</v>
+        <v>0.003121058211573426</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.8575757575758</v>
+        <v>386.7848484848485</v>
       </c>
       <c r="B49">
-        <v>0.002961492455503649</v>
+        <v>0.003047624334014674</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.9545454545455</v>
+        <v>394.7909090909091</v>
       </c>
       <c r="B50">
-        <v>0.002888559302845906</v>
+        <v>0.002977370324925316</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>408.0515151515152</v>
+        <v>402.7969696969697</v>
       </c>
       <c r="B51">
-        <v>0.002818830749954937</v>
+        <v>0.002910098106220766</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>416.1484848484849</v>
+        <v>410.8030303030303</v>
       </c>
       <c r="B52">
-        <v>0.002752106507966855</v>
+        <v>0.002845625553184896</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>424.2454545454546</v>
+        <v>418.8090909090909</v>
       </c>
       <c r="B53">
-        <v>0.002688202382178486</v>
+        <v>0.002783784929549944</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>432.3424242424243</v>
+        <v>426.8151515151515</v>
       </c>
       <c r="B54">
-        <v>0.002626948702199065</v>
+        <v>0.002724421502523833</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.439393939394</v>
+        <v>434.8212121212121</v>
       </c>
       <c r="B55">
-        <v>0.002568188931217557</v>
+        <v>0.002667392314144691</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.5363636363637</v>
+        <v>442.8272727272727</v>
       </c>
       <c r="B56">
-        <v>0.00251177843109041</v>
+        <v>0.00261256508881331</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.6333333333334</v>
+        <v>450.8333333333333</v>
       </c>
       <c r="B57">
-        <v>0.002457583363342884</v>
+        <v>0.00255981725976266</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.7303030303031</v>
+        <v>458.8393939393939</v>
       </c>
       <c r="B58">
-        <v>0.002405479709022215</v>
+        <v>0.002509035099668747</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.8272727272728</v>
+        <v>466.8454545454545</v>
       </c>
       <c r="B59">
-        <v>0.002355352392737675</v>
+        <v>0.002460112942669601</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.9242424242425</v>
+        <v>474.8515151515151</v>
       </c>
       <c r="B60">
-        <v>0.002307094498248114</v>
+        <v>0.002412952486804241</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>489.0212121212122</v>
+        <v>482.8575757575758</v>
       </c>
       <c r="B61">
-        <v>0.00226060656467445</v>
+        <v>0.002367462167364444</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>497.1181818181819</v>
+        <v>490.8636363636364</v>
       </c>
       <c r="B62">
-        <v>0.00221579595387411</v>
+        <v>0.002323556592912663</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>505.2151515151515</v>
+        <v>498.869696969697</v>
       </c>
       <c r="B63">
-        <v>0.002172576280758743</v>
+        <v>0.002281156036795257</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>513.3121212121213</v>
+        <v>506.8757575757576</v>
       </c>
       <c r="B64">
-        <v>0.002130866899400167</v>
+        <v>0.002240185977900962</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>521.4090909090909</v>
+        <v>514.8818181818182</v>
       </c>
       <c r="B65">
-        <v>0.00209059243868117</v>
+        <v>0.002200576685204554</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>529.5060606060606</v>
+        <v>522.8878787878788</v>
       </c>
       <c r="B66">
-        <v>0.002051682382031121</v>
+        <v>0.002162262841315321</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>537.6030303030303</v>
+        <v>530.8939393939394</v>
       </c>
       <c r="B67">
-        <v>0.002014070686461129</v>
+        <v>0.002125183200835971</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.7</v>
+        <v>538.9</v>
       </c>
       <c r="B68">
-        <v>0.001977695436696093</v>
+        <v>0.002089280279844253</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.7969696969697</v>
+        <v>546.9060606060606</v>
       </c>
       <c r="B69">
-        <v>0.001942498530705191</v>
+        <v>0.002054500073248407</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.8939393939394</v>
+        <v>554.9121212121212</v>
       </c>
       <c r="B70">
-        <v>0.001908425393369704</v>
+        <v>0.002020791797148658</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.9909090909091</v>
+        <v>562.9181818181818</v>
       </c>
       <c r="B71">
-        <v>0.001875424715407219</v>
+        <v>0.001988107653668595</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>578.0878787878788</v>
+        <v>570.9242424242424</v>
       </c>
       <c r="B72">
-        <v>0.001843448215002397</v>
+        <v>0.001956402616009377</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>586.1848484848484</v>
+        <v>578.930303030303</v>
       </c>
       <c r="B73">
-        <v>0.001812450419883519</v>
+        <v>0.001925634231732409</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>594.2818181818182</v>
+        <v>586.9363636363636</v>
       </c>
       <c r="B74">
-        <v>0.001782388467836827</v>
+        <v>0.00189576244249727</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>602.3787878787879</v>
+        <v>594.9424242424242</v>
       </c>
       <c r="B75">
-        <v>0.001753221923872184</v>
+        <v>0.001866749418675721</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>610.4757575757576</v>
+        <v>602.9484848484848</v>
       </c>
       <c r="B76">
-        <v>0.001724912612448014</v>
+        <v>0.001838559407433083</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>618.5727272727273</v>
+        <v>610.9545454545455</v>
       </c>
       <c r="B77">
-        <v>0.001697424463334556</v>
+        <v>0.00181115859301838</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>626.6696969696969</v>
+        <v>618.9606060606061</v>
       </c>
       <c r="B78">
-        <v>0.00167072336984511</v>
+        <v>0.001784514968137032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>634.7666666666667</v>
+        <v>626.9666666666667</v>
       </c>
       <c r="B79">
-        <v>0.00164477705829798</v>
+        <v>0.001758598215396764</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>642.8636363636364</v>
+        <v>634.9727272727273</v>
       </c>
       <c r="B80">
-        <v>0.001619554967689372</v>
+        <v>0.001733379597920934</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.9606060606061</v>
+        <v>642.9787878787879</v>
       </c>
       <c r="B81">
-        <v>0.001595028138661609</v>
+        <v>0.001708831858315155</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>659.0575757575757</v>
+        <v>650.9848484848485</v>
       </c>
       <c r="B82">
-        <v>0.001571169110943376</v>
+        <v>0.001684929125254508</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>667.1545454545454</v>
+        <v>658.9909090909091</v>
       </c>
       <c r="B83">
-        <v>0.001547951828520692</v>
+        <v>0.001661646827031027</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>675.2515151515152</v>
+        <v>666.9969696969697</v>
       </c>
       <c r="B84">
-        <v>0.001525351551870314</v>
+        <v>0.001638961611465592</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>683.3484848484849</v>
+        <v>675.0030303030303</v>
       </c>
       <c r="B85">
-        <v>0.001503344776652226</v>
+        <v>0.001616851271645816</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>691.4454545454546</v>
+        <v>683.0090909090909</v>
       </c>
       <c r="B86">
-        <v>0.001481909158315892</v>
+        <v>0.001595294677002861</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>699.5424242424242</v>
+        <v>691.0151515151515</v>
       </c>
       <c r="B87">
-        <v>0.001461023442126762</v>
+        <v>0.001574271709285973</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>707.6393939393939</v>
+        <v>699.0212121212121</v>
       </c>
       <c r="B88">
-        <v>0.001440667398165869</v>
+        <v>0.001553763203034644</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>715.7363636363636</v>
+        <v>707.0272727272727</v>
       </c>
       <c r="B89">
-        <v>0.001420821760896863</v>
+        <v>0.001533750890185145</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>723.8333333333334</v>
+        <v>715.0333333333333</v>
       </c>
       <c r="B90">
-        <v>0.001401468172932123</v>
+        <v>0.001514217348481232</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>731.9303030303031</v>
+        <v>723.0393939393939</v>
       </c>
       <c r="B91">
-        <v>0.001382589132662983</v>
+        <v>0.001495145953388581</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>740.0272727272727</v>
+        <v>731.0454545454545</v>
       </c>
       <c r="B92">
-        <v>0.001364167945449245</v>
+        <v>0.001476520833239256</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>748.1242424242424</v>
+        <v>739.0515151515151</v>
       </c>
       <c r="B93">
-        <v>0.001346188678090202</v>
+        <v>0.00145832682735662</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>756.2212121212121</v>
+        <v>747.0575757575757</v>
       </c>
       <c r="B94">
-        <v>0.001328636116323822</v>
+        <v>0.001440549446932866</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>764.3181818181819</v>
+        <v>755.0636363636363</v>
       </c>
       <c r="B95">
-        <v>0.001311495725122791</v>
+        <v>0.001423174838450966</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>772.4151515151515</v>
+        <v>763.0696969696969</v>
       </c>
       <c r="B96">
-        <v>0.00129475361157598</v>
+        <v>0.001406189749460629</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>780.5121212121212</v>
+        <v>771.0757575757575</v>
       </c>
       <c r="B97">
-        <v>0.001278396490161965</v>
+        <v>0.001389581496533911</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>788.6090909090909</v>
+        <v>779.0818181818181</v>
       </c>
       <c r="B98">
-        <v>0.001262411650237472</v>
+        <v>0.00137333793524071</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>796.7060606060606</v>
+        <v>787.0878787878788</v>
       </c>
       <c r="B99">
-        <v>0.001246786925578432</v>
+        <v>0.001357447431997586</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>804.8030303030304</v>
+        <v>795.0939393939394</v>
       </c>
       <c r="B100">
-        <v>0.001231510665824734</v>
+        <v>0.00134189883765535</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="B101">
-        <v>0.001216571709691934</v>
+        <v>0.00132668146270177</v>
       </c>
     </row>
   </sheetData>
@@ -2720,25 +2720,25 @@
         <v>62</v>
       </c>
       <c r="B2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="C2">
-        <v>1.3</v>
+        <v>1.408308678285174</v>
       </c>
       <c r="D2">
-        <v>0.223665</v>
+        <v>0.185419</v>
       </c>
       <c r="E2">
-        <v>0.08689313063566455</v>
+        <v>0.02764825308727077</v>
       </c>
       <c r="F2">
-        <v>1.05307844348342</v>
+        <v>1.021189299069938</v>
       </c>
       <c r="G2">
-        <v>-0.6504019707362143</v>
+        <v>-0.7318457654861891</v>
       </c>
       <c r="H2">
-        <v>-0.7360841467267152</v>
+        <v>-0.7956170590946079</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -2746,25 +2746,25 @@
         <v>125</v>
       </c>
       <c r="B3">
-        <v>39</v>
+        <v>38.1</v>
       </c>
       <c r="C3">
-        <v>3.0840089349921</v>
+        <v>1.27758452644912</v>
       </c>
       <c r="D3">
-        <v>0.047857</v>
+        <v>0.03847</v>
       </c>
       <c r="E3">
-        <v>0.005268825939218126</v>
+        <v>0.003421588649865569</v>
       </c>
       <c r="F3">
-        <v>1.591064607026499</v>
+        <v>1.580924975675619</v>
       </c>
       <c r="G3">
-        <v>-1.320054529380785</v>
+        <v>-1.414877813693185</v>
       </c>
       <c r="H3">
-        <v>-1.299983122420791</v>
+        <v>-1.347299254247706</v>
       </c>
     </row>
     <row r="4" spans="1:8">
@@ -2772,25 +2772,25 @@
         <v>188</v>
       </c>
       <c r="B4">
-        <v>79.09999999999999</v>
+        <v>81</v>
       </c>
       <c r="C4">
-        <v>2.478574859336174</v>
+        <v>2.394437999475729</v>
       </c>
       <c r="D4">
-        <v>0.01952</v>
+        <v>0.018984</v>
       </c>
       <c r="E4">
-        <v>0.001232376205187</v>
+        <v>0.00127096481287074</v>
       </c>
       <c r="F4">
-        <v>1.898176483497676</v>
+        <v>1.90848501887865</v>
       </c>
       <c r="G4">
-        <v>-1.709520186669327</v>
+        <v>-1.721612274790717</v>
       </c>
       <c r="H4">
-        <v>-1.621887446920606</v>
+        <v>-1.670146360893718</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -2798,25 +2798,25 @@
         <v>251</v>
       </c>
       <c r="B5">
-        <v>130.9</v>
+        <v>137.5</v>
       </c>
       <c r="C5">
-        <v>4.787599723359411</v>
+        <v>4.185291706281256</v>
       </c>
       <c r="D5">
-        <v>0.012653</v>
+        <v>0.012357</v>
       </c>
       <c r="E5">
-        <v>0.001167132335636747</v>
+        <v>0.0007632111255886026</v>
       </c>
       <c r="F5">
-        <v>2.116939646550756</v>
+        <v>2.138302698166282</v>
       </c>
       <c r="G5">
-        <v>-1.897806491960256</v>
+        <v>-1.90808695332392</v>
       </c>
       <c r="H5">
-        <v>-1.851187625856062</v>
+        <v>-1.896657421548708</v>
       </c>
     </row>
     <row r="6" spans="1:8">
@@ -2824,25 +2824,25 @@
         <v>314</v>
       </c>
       <c r="B6">
-        <v>214.1</v>
+        <v>211.1</v>
       </c>
       <c r="C6">
-        <v>4.670117771534247</v>
+        <v>5.722179072113467</v>
       </c>
       <c r="D6">
-        <v>0.007606</v>
+        <v>0.008705000000000001</v>
       </c>
       <c r="E6">
-        <v>0.000416579190817571</v>
+        <v>0.0005302289861727458</v>
       </c>
       <c r="F6">
-        <v>2.330616667294438</v>
+        <v>2.324488233307656</v>
       </c>
       <c r="G6">
-        <v>-2.118843678924436</v>
+        <v>-2.06023122454665</v>
       </c>
       <c r="H6">
-        <v>-2.075156681738808</v>
+        <v>-2.080164117701128</v>
       </c>
     </row>
     <row r="7" spans="1:8">
@@ -2850,25 +2850,25 @@
         <v>376</v>
       </c>
       <c r="B7">
-        <v>288.1</v>
+        <v>287.4</v>
       </c>
       <c r="C7">
-        <v>5.685165882462103</v>
+        <v>3.679371927079101</v>
       </c>
       <c r="D7">
-        <v>0.00615</v>
+        <v>0.006292000000000001</v>
       </c>
       <c r="E7">
-        <v>0.0003635351121663185</v>
+        <v>0.0001936308056299124</v>
       </c>
       <c r="F7">
-        <v>2.459543258280413</v>
+        <v>2.458486763798207</v>
       </c>
       <c r="G7">
-        <v>-2.211124884224583</v>
+        <v>-2.201211286048751</v>
       </c>
       <c r="H7">
-        <v>-2.210293191789403</v>
+        <v>-2.212234676248701</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -2876,25 +2876,25 @@
         <v>439</v>
       </c>
       <c r="B8">
-        <v>394</v>
+        <v>393.5</v>
       </c>
       <c r="C8">
-        <v>3.346640106136302</v>
+        <v>5.066776314603025</v>
       </c>
       <c r="D8">
-        <v>0.004235000000000001</v>
+        <v>0.004414</v>
       </c>
       <c r="E8">
-        <v>0.0001603347193287288</v>
+        <v>0.0002112144776182626</v>
       </c>
       <c r="F8">
-        <v>2.595496221825574</v>
+        <v>2.594944736695084</v>
       </c>
       <c r="G8">
-        <v>-2.373146585333274</v>
+        <v>-2.355167671174364</v>
       </c>
       <c r="H8">
-        <v>-2.352794508887963</v>
+        <v>-2.346729290725321</v>
       </c>
     </row>
     <row r="9" spans="1:8">
@@ -2902,25 +2902,25 @@
         <v>502</v>
       </c>
       <c r="B9">
-        <v>515.2</v>
+        <v>515.3</v>
       </c>
       <c r="C9">
-        <v>3.805843460317889</v>
+        <v>7.935923946768195</v>
       </c>
       <c r="D9">
-        <v>0.003294</v>
+        <v>0.003261</v>
       </c>
       <c r="E9">
-        <v>0.0001124000790826136</v>
+        <v>0.0001578497879490358</v>
       </c>
       <c r="F9">
-        <v>2.711975854351756</v>
+        <v>2.712060142461075</v>
       </c>
       <c r="G9">
-        <v>-2.482276405166265</v>
+        <v>-2.486649201194043</v>
       </c>
       <c r="H9">
-        <v>-2.474884536330605</v>
+        <v>-2.462159639083738</v>
       </c>
     </row>
     <row r="10" spans="1:8">
@@ -2928,25 +2928,25 @@
         <v>565</v>
       </c>
       <c r="B10">
-        <v>662.5</v>
+        <v>665.3</v>
       </c>
       <c r="C10">
-        <v>6.057593948462082</v>
+        <v>8.203048213926333</v>
       </c>
       <c r="D10">
-        <v>0.002638000000000001</v>
+        <v>0.002514</v>
       </c>
       <c r="E10">
-        <v>7.209253313161726E-05</v>
+        <v>0.0001025367142918954</v>
       </c>
       <c r="F10">
-        <v>2.821185882608845</v>
+        <v>2.823017523446049</v>
       </c>
       <c r="G10">
-        <v>-2.578725208789654</v>
+        <v>-2.599634726650061</v>
       </c>
       <c r="H10">
-        <v>-2.589354809439706</v>
+        <v>-2.571520564371608</v>
       </c>
     </row>
     <row r="11" spans="1:8">
@@ -2954,25 +2954,25 @@
         <v>628</v>
       </c>
       <c r="B11">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="C11">
-        <v>9.599131905195039</v>
+        <v>7.651361534611556</v>
       </c>
       <c r="D11">
-        <v>0.00213</v>
+        <v>0.002173</v>
       </c>
       <c r="E11">
-        <v>6.881537295950343E-05</v>
+        <v>6.824872811187685E-05</v>
       </c>
       <c r="F11">
-        <v>2.910037123553051</v>
+        <v>2.904769625906595</v>
       </c>
       <c r="G11">
-        <v>-2.671620396561262</v>
+        <v>-2.662940273679475</v>
       </c>
       <c r="H11">
-        <v>-2.68248568743035</v>
+        <v>-2.652096416919216</v>
       </c>
     </row>
     <row r="12" spans="1:8">
@@ -2998,7 +2998,7 @@
         <v>-2.338187314462739</v>
       </c>
       <c r="H12">
-        <v>-2.457595894667791</v>
+        <v>-2.445819704215646</v>
       </c>
     </row>
   </sheetData>
@@ -3021,802 +3021,802 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2">
-        <v>11.3</v>
+        <v>10.5</v>
       </c>
       <c r="B2">
-        <v>0.2234229411226657</v>
+        <v>0.184891647846076</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3">
-        <v>19.3969696969697</v>
+        <v>18.50606060606061</v>
       </c>
       <c r="B3">
-        <v>0.1156212373834673</v>
+        <v>0.09699386650165555</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4">
-        <v>27.4939393939394</v>
+        <v>26.51212121212121</v>
       </c>
       <c r="B4">
-        <v>0.07556595810281702</v>
+        <v>0.06441915600835781</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5">
-        <v>35.59090909090909</v>
+        <v>34.51818181818182</v>
       </c>
       <c r="B5">
-        <v>0.05516354196624016</v>
+        <v>0.04770430921186292</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
-        <v>43.68787878787879</v>
+        <v>42.52424242424242</v>
       </c>
       <c r="B6">
-        <v>0.04296524975839557</v>
+        <v>0.03762158624308524</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>51.78484848484848</v>
+        <v>50.53030303030303</v>
       </c>
       <c r="B7">
-        <v>0.03492127028347099</v>
+        <v>0.03091421103869369</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>59.88181818181819</v>
+        <v>58.53636363636363</v>
       </c>
       <c r="B8">
-        <v>0.02925286548600948</v>
+        <v>0.02614858339296097</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9">
-        <v>67.97878787878788</v>
+        <v>66.54242424242423</v>
       </c>
       <c r="B9">
-        <v>0.02506208489084306</v>
+        <v>0.02259818839391243</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>76.07575757575758</v>
+        <v>74.54848484848485</v>
       </c>
       <c r="B10">
-        <v>0.02184900993129131</v>
+        <v>0.01985673358482553</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>84.17272727272727</v>
+        <v>82.55454545454545</v>
       </c>
       <c r="B11">
-        <v>0.01931428318245793</v>
+        <v>0.01767978487064297</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12">
-        <v>92.26969696969697</v>
+        <v>90.56060606060606</v>
       </c>
       <c r="B12">
-        <v>0.01726822968450587</v>
+        <v>0.01591174092637995</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13">
-        <v>100.3666666666667</v>
+        <v>98.56666666666666</v>
       </c>
       <c r="B13">
-        <v>0.01558512248656729</v>
+        <v>0.01444898696256113</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14">
-        <v>108.4636363636364</v>
+        <v>106.5727272727273</v>
       </c>
       <c r="B14">
-        <v>0.01417848879016148</v>
+        <v>0.01321994121343388</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15">
-        <v>116.5606060606061</v>
+        <v>114.5787878787879</v>
       </c>
       <c r="B15">
-        <v>0.01298699511530168</v>
+        <v>0.01217361410153211</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16">
-        <v>124.6575757575758</v>
+        <v>122.5848484848485</v>
       </c>
       <c r="B16">
-        <v>0.01196599002919759</v>
+        <v>0.01127273135110265</v>
       </c>
     </row>
     <row r="17" spans="1:2">
       <c r="A17">
-        <v>132.7545454545455</v>
+        <v>130.5909090909091</v>
       </c>
       <c r="B17">
-        <v>0.0110822316650582</v>
+        <v>0.01048943309212318</v>
       </c>
     </row>
     <row r="18" spans="1:2">
       <c r="A18">
-        <v>140.8515151515152</v>
+        <v>138.5969696969697</v>
       </c>
       <c r="B18">
-        <v>0.01031048744007662</v>
+        <v>0.009802491403436467</v>
       </c>
     </row>
     <row r="19" spans="1:2">
       <c r="A19">
-        <v>148.9484848484849</v>
+        <v>146.6030303030303</v>
       </c>
       <c r="B19">
-        <v>0.009631275999786809</v>
+        <v>0.009195456799216902</v>
       </c>
     </row>
     <row r="20" spans="1:2">
       <c r="A20">
-        <v>157.0454545454546</v>
+        <v>154.6090909090909</v>
       </c>
       <c r="B20">
-        <v>0.009029328839544866</v>
+        <v>0.008655391614442896</v>
       </c>
     </row>
     <row r="21" spans="1:2">
       <c r="A21">
-        <v>165.1424242424243</v>
+        <v>162.6151515151515</v>
       </c>
       <c r="B21">
-        <v>0.008492518339989152</v>
+        <v>0.008171984784864205</v>
       </c>
     </row>
     <row r="22" spans="1:2">
       <c r="A22">
-        <v>173.2393939393939</v>
+        <v>170.6212121212121</v>
       </c>
       <c r="B22">
-        <v>0.008011095705198019</v>
+        <v>0.007736920717535016</v>
       </c>
     </row>
     <row r="23" spans="1:2">
       <c r="A23">
-        <v>181.3363636363637</v>
+        <v>178.6272727272727</v>
       </c>
       <c r="B23">
-        <v>0.007577139428687919</v>
+        <v>0.007343421227736977</v>
       </c>
     </row>
     <row r="24" spans="1:2">
       <c r="A24">
-        <v>189.4333333333334</v>
+        <v>186.6333333333333</v>
       </c>
       <c r="B24">
-        <v>0.007184149648374311</v>
+        <v>0.006985907714317893</v>
       </c>
     </row>
     <row r="25" spans="1:2">
       <c r="A25">
-        <v>197.5303030303031</v>
+        <v>194.6393939393939</v>
       </c>
       <c r="B25">
-        <v>0.006826745424516108</v>
+        <v>0.006659748375801701</v>
       </c>
     </row>
     <row r="26" spans="1:2">
       <c r="A26">
-        <v>205.6272727272728</v>
+        <v>202.6454545454545</v>
       </c>
       <c r="B26">
-        <v>0.006500435816382649</v>
+        <v>0.006361066553561816</v>
       </c>
     </row>
     <row r="27" spans="1:2">
       <c r="A27">
-        <v>213.7242424242424</v>
+        <v>210.6515151515152</v>
       </c>
       <c r="B27">
-        <v>0.006201444662158525</v>
+        <v>0.006086593664304345</v>
       </c>
     </row>
     <row r="28" spans="1:2">
       <c r="A28">
-        <v>221.8212121212121</v>
+        <v>218.6575757575758</v>
       </c>
       <c r="B28">
-        <v>0.005926574970018011</v>
+        <v>0.005833555098793225</v>
       </c>
     </row>
     <row r="29" spans="1:2">
       <c r="A29">
-        <v>229.9181818181818</v>
+        <v>226.6636363636364</v>
       </c>
       <c r="B29">
-        <v>0.00567310289062023</v>
+        <v>0.005599580796224393</v>
       </c>
     </row>
     <row r="30" spans="1:2">
       <c r="A30">
-        <v>238.0151515151516</v>
+        <v>234.669696969697</v>
       </c>
       <c r="B30">
-        <v>0.005438694034608454</v>
+        <v>0.005382634499791695</v>
       </c>
     </row>
     <row r="31" spans="1:2">
       <c r="A31">
-        <v>246.1121212121213</v>
+        <v>242.6757575757576</v>
       </c>
       <c r="B31">
-        <v>0.00522133684803717</v>
+        <v>0.005180957304561919</v>
       </c>
     </row>
     <row r="32" spans="1:2">
       <c r="A32">
-        <v>254.2090909090909</v>
+        <v>250.6818181818182</v>
       </c>
       <c r="B32">
-        <v>0.005019289137692525</v>
+        <v>0.004993022246858652</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="A33">
-        <v>262.3060606060606</v>
+        <v>258.6878787878788</v>
       </c>
       <c r="B33">
-        <v>0.004831034826267896</v>
+        <v>0.004817497501294103</v>
       </c>
     </row>
     <row r="34" spans="1:2">
       <c r="A34">
-        <v>270.4030303030303</v>
+        <v>266.6939393939394</v>
       </c>
       <c r="B34">
-        <v>0.0046552487335509</v>
+        <v>0.004653216344908505</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35">
-        <v>278.5000000000001</v>
+        <v>274.7</v>
       </c>
       <c r="B35">
-        <v>0.004490767704652825</v>
+        <v>0.004499152483511465</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="A36">
-        <v>286.5969696969697</v>
+        <v>282.7060606060606</v>
       </c>
       <c r="B36">
-        <v>0.004336566794921568</v>
+        <v>0.00435439965844809</v>
       </c>
     </row>
     <row r="37" spans="1:2">
       <c r="A37">
-        <v>294.6939393939394</v>
+        <v>290.7121212121212</v>
       </c>
       <c r="B37">
-        <v>0.004191739511663775</v>
+        <v>0.004218154693983959</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38">
-        <v>302.7909090909091</v>
+        <v>298.7181818181818</v>
       </c>
       <c r="B38">
-        <v>0.004055481331892936</v>
+        <v>0.004089703328325833</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="A39">
-        <v>310.8878787878788</v>
+        <v>306.7242424242424</v>
       </c>
       <c r="B39">
-        <v>0.003927075881962371</v>
+        <v>0.003968408310592312</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="A40">
-        <v>318.9848484848485</v>
+        <v>314.730303030303</v>
       </c>
       <c r="B40">
-        <v>0.003805883292700867</v>
+        <v>0.003853699353024394</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="A41">
-        <v>327.0818181818182</v>
+        <v>322.7363636363636</v>
       </c>
       <c r="B41">
-        <v>0.003691330342352621</v>
+        <v>0.003745064610494677</v>
       </c>
     </row>
     <row r="42" spans="1:2">
       <c r="A42">
-        <v>335.1787878787879</v>
+        <v>330.7424242424242</v>
       </c>
       <c r="B42">
-        <v>0.00358290207638999</v>
+        <v>0.003642043423865678</v>
       </c>
     </row>
     <row r="43" spans="1:2">
       <c r="A43">
-        <v>343.2757575757576</v>
+        <v>338.7484848484848</v>
       </c>
       <c r="B43">
-        <v>0.003480134653385886</v>
+        <v>0.003544220114334572</v>
       </c>
     </row>
     <row r="44" spans="1:2">
       <c r="A44">
-        <v>351.3727272727273</v>
+        <v>346.7545454545455</v>
       </c>
       <c r="B44">
-        <v>0.003382609213512734</v>
+        <v>0.003451218655832776</v>
       </c>
     </row>
     <row r="45" spans="1:2">
       <c r="A45">
-        <v>359.469696969697</v>
+        <v>354.7606060606061</v>
       </c>
       <c r="B45">
-        <v>0.003289946603801274</v>
+        <v>0.003362698084258411</v>
       </c>
     </row>
     <row r="46" spans="1:2">
       <c r="A46">
-        <v>367.5666666666667</v>
+        <v>362.7666666666667</v>
       </c>
       <c r="B46">
-        <v>0.003201802824248834</v>
+        <v>0.003278348527644262</v>
       </c>
     </row>
     <row r="47" spans="1:2">
       <c r="A47">
-        <v>375.6636363636364</v>
+        <v>370.7727272727273</v>
       </c>
       <c r="B47">
-        <v>0.003117865082885064</v>
+        <v>0.003197887761699077</v>
       </c>
     </row>
     <row r="48" spans="1:2">
       <c r="A48">
-        <v>383.7606060606061</v>
+        <v>378.7787878787879</v>
       </c>
       <c r="B48">
-        <v>0.003037848367260696</v>
+        <v>0.003121058211573426</v>
       </c>
     </row>
     <row r="49" spans="1:2">
       <c r="A49">
-        <v>391.8575757575758</v>
+        <v>386.7848484848485</v>
       </c>
       <c r="B49">
-        <v>0.002961492455503649</v>
+        <v>0.003047624334014674</v>
       </c>
     </row>
     <row r="50" spans="1:2">
       <c r="A50">
-        <v>399.9545454545455</v>
+        <v>394.7909090909091</v>
       </c>
       <c r="B50">
-        <v>0.002888559302845906</v>
+        <v>0.002977370324925316</v>
       </c>
     </row>
     <row r="51" spans="1:2">
       <c r="A51">
-        <v>408.0515151515152</v>
+        <v>402.7969696969697</v>
       </c>
       <c r="B51">
-        <v>0.002818830749954937</v>
+        <v>0.002910098106220766</v>
       </c>
     </row>
     <row r="52" spans="1:2">
       <c r="A52">
-        <v>416.1484848484849</v>
+        <v>410.8030303030303</v>
       </c>
       <c r="B52">
-        <v>0.002752106507966855</v>
+        <v>0.002845625553184896</v>
       </c>
     </row>
     <row r="53" spans="1:2">
       <c r="A53">
-        <v>424.2454545454546</v>
+        <v>418.8090909090909</v>
       </c>
       <c r="B53">
-        <v>0.002688202382178486</v>
+        <v>0.002783784929549944</v>
       </c>
     </row>
     <row r="54" spans="1:2">
       <c r="A54">
-        <v>432.3424242424243</v>
+        <v>426.8151515151515</v>
       </c>
       <c r="B54">
-        <v>0.002626948702199065</v>
+        <v>0.002724421502523833</v>
       </c>
     </row>
     <row r="55" spans="1:2">
       <c r="A55">
-        <v>440.439393939394</v>
+        <v>434.8212121212121</v>
       </c>
       <c r="B55">
-        <v>0.002568188931217557</v>
+        <v>0.002667392314144691</v>
       </c>
     </row>
     <row r="56" spans="1:2">
       <c r="A56">
-        <v>448.5363636363637</v>
+        <v>442.8272727272727</v>
       </c>
       <c r="B56">
-        <v>0.00251177843109041</v>
+        <v>0.00261256508881331</v>
       </c>
     </row>
     <row r="57" spans="1:2">
       <c r="A57">
-        <v>456.6333333333334</v>
+        <v>450.8333333333333</v>
       </c>
       <c r="B57">
-        <v>0.002457583363342884</v>
+        <v>0.00255981725976266</v>
       </c>
     </row>
     <row r="58" spans="1:2">
       <c r="A58">
-        <v>464.7303030303031</v>
+        <v>458.8393939393939</v>
       </c>
       <c r="B58">
-        <v>0.002405479709022215</v>
+        <v>0.002509035099668747</v>
       </c>
     </row>
     <row r="59" spans="1:2">
       <c r="A59">
-        <v>472.8272727272728</v>
+        <v>466.8454545454545</v>
       </c>
       <c r="B59">
-        <v>0.002355352392737675</v>
+        <v>0.002460112942669601</v>
       </c>
     </row>
     <row r="60" spans="1:2">
       <c r="A60">
-        <v>480.9242424242425</v>
+        <v>474.8515151515151</v>
       </c>
       <c r="B60">
-        <v>0.002307094498248114</v>
+        <v>0.002412952486804241</v>
       </c>
     </row>
     <row r="61" spans="1:2">
       <c r="A61">
-        <v>489.0212121212122</v>
+        <v>482.8575757575758</v>
       </c>
       <c r="B61">
-        <v>0.00226060656467445</v>
+        <v>0.002367462167364444</v>
       </c>
     </row>
     <row r="62" spans="1:2">
       <c r="A62">
-        <v>497.1181818181819</v>
+        <v>490.8636363636364</v>
       </c>
       <c r="B62">
-        <v>0.00221579595387411</v>
+        <v>0.002323556592912663</v>
       </c>
     </row>
     <row r="63" spans="1:2">
       <c r="A63">
-        <v>505.2151515151515</v>
+        <v>498.869696969697</v>
       </c>
       <c r="B63">
-        <v>0.002172576280758743</v>
+        <v>0.002281156036795257</v>
       </c>
     </row>
     <row r="64" spans="1:2">
       <c r="A64">
-        <v>513.3121212121213</v>
+        <v>506.8757575757576</v>
       </c>
       <c r="B64">
-        <v>0.002130866899400167</v>
+        <v>0.002240185977900962</v>
       </c>
     </row>
     <row r="65" spans="1:2">
       <c r="A65">
-        <v>521.4090909090909</v>
+        <v>514.8818181818182</v>
       </c>
       <c r="B65">
-        <v>0.00209059243868117</v>
+        <v>0.002200576685204554</v>
       </c>
     </row>
     <row r="66" spans="1:2">
       <c r="A66">
-        <v>529.5060606060606</v>
+        <v>522.8878787878788</v>
       </c>
       <c r="B66">
-        <v>0.002051682382031121</v>
+        <v>0.002162262841315321</v>
       </c>
     </row>
     <row r="67" spans="1:2">
       <c r="A67">
-        <v>537.6030303030303</v>
+        <v>530.8939393939394</v>
       </c>
       <c r="B67">
-        <v>0.002014070686461129</v>
+        <v>0.002125183200835971</v>
       </c>
     </row>
     <row r="68" spans="1:2">
       <c r="A68">
-        <v>545.7</v>
+        <v>538.9</v>
       </c>
       <c r="B68">
-        <v>0.001977695436696093</v>
+        <v>0.002089280279844253</v>
       </c>
     </row>
     <row r="69" spans="1:2">
       <c r="A69">
-        <v>553.7969696969697</v>
+        <v>546.9060606060606</v>
       </c>
       <c r="B69">
-        <v>0.001942498530705191</v>
+        <v>0.002054500073248407</v>
       </c>
     </row>
     <row r="70" spans="1:2">
       <c r="A70">
-        <v>561.8939393939394</v>
+        <v>554.9121212121212</v>
       </c>
       <c r="B70">
-        <v>0.001908425393369704</v>
+        <v>0.002020791797148658</v>
       </c>
     </row>
     <row r="71" spans="1:2">
       <c r="A71">
-        <v>569.9909090909091</v>
+        <v>562.9181818181818</v>
       </c>
       <c r="B71">
-        <v>0.001875424715407219</v>
+        <v>0.001988107653668595</v>
       </c>
     </row>
     <row r="72" spans="1:2">
       <c r="A72">
-        <v>578.0878787878788</v>
+        <v>570.9242424242424</v>
       </c>
       <c r="B72">
-        <v>0.001843448215002397</v>
+        <v>0.001956402616009377</v>
       </c>
     </row>
     <row r="73" spans="1:2">
       <c r="A73">
-        <v>586.1848484848484</v>
+        <v>578.930303030303</v>
       </c>
       <c r="B73">
-        <v>0.001812450419883519</v>
+        <v>0.001925634231732409</v>
       </c>
     </row>
     <row r="74" spans="1:2">
       <c r="A74">
-        <v>594.2818181818182</v>
+        <v>586.9363636363636</v>
       </c>
       <c r="B74">
-        <v>0.001782388467836827</v>
+        <v>0.00189576244249727</v>
       </c>
     </row>
     <row r="75" spans="1:2">
       <c r="A75">
-        <v>602.3787878787879</v>
+        <v>594.9424242424242</v>
       </c>
       <c r="B75">
-        <v>0.001753221923872184</v>
+        <v>0.001866749418675721</v>
       </c>
     </row>
     <row r="76" spans="1:2">
       <c r="A76">
-        <v>610.4757575757576</v>
+        <v>602.9484848484848</v>
       </c>
       <c r="B76">
-        <v>0.001724912612448014</v>
+        <v>0.001838559407433083</v>
       </c>
     </row>
     <row r="77" spans="1:2">
       <c r="A77">
-        <v>618.5727272727273</v>
+        <v>610.9545454545455</v>
       </c>
       <c r="B77">
-        <v>0.001697424463334556</v>
+        <v>0.00181115859301838</v>
       </c>
     </row>
     <row r="78" spans="1:2">
       <c r="A78">
-        <v>626.6696969696969</v>
+        <v>618.9606060606061</v>
       </c>
       <c r="B78">
-        <v>0.00167072336984511</v>
+        <v>0.001784514968137032</v>
       </c>
     </row>
     <row r="79" spans="1:2">
       <c r="A79">
-        <v>634.7666666666667</v>
+        <v>626.9666666666667</v>
       </c>
       <c r="B79">
-        <v>0.00164477705829798</v>
+        <v>0.001758598215396764</v>
       </c>
     </row>
     <row r="80" spans="1:2">
       <c r="A80">
-        <v>642.8636363636364</v>
+        <v>634.9727272727273</v>
       </c>
       <c r="B80">
-        <v>0.001619554967689372</v>
+        <v>0.001733379597920934</v>
       </c>
     </row>
     <row r="81" spans="1:2">
       <c r="A81">
-        <v>650.9606060606061</v>
+        <v>642.9787878787879</v>
       </c>
       <c r="B81">
-        <v>0.001595028138661609</v>
+        <v>0.001708831858315155</v>
       </c>
     </row>
     <row r="82" spans="1:2">
       <c r="A82">
-        <v>659.0575757575757</v>
+        <v>650.9848484848485</v>
       </c>
       <c r="B82">
-        <v>0.001571169110943376</v>
+        <v>0.001684929125254508</v>
       </c>
     </row>
     <row r="83" spans="1:2">
       <c r="A83">
-        <v>667.1545454545454</v>
+        <v>658.9909090909091</v>
       </c>
       <c r="B83">
-        <v>0.001547951828520692</v>
+        <v>0.001661646827031027</v>
       </c>
     </row>
     <row r="84" spans="1:2">
       <c r="A84">
-        <v>675.2515151515152</v>
+        <v>666.9969696969697</v>
       </c>
       <c r="B84">
-        <v>0.001525351551870314</v>
+        <v>0.001638961611465592</v>
       </c>
     </row>
     <row r="85" spans="1:2">
       <c r="A85">
-        <v>683.3484848484849</v>
+        <v>675.0030303030303</v>
       </c>
       <c r="B85">
-        <v>0.001503344776652226</v>
+        <v>0.001616851271645816</v>
       </c>
     </row>
     <row r="86" spans="1:2">
       <c r="A86">
-        <v>691.4454545454546</v>
+        <v>683.0090909090909</v>
       </c>
       <c r="B86">
-        <v>0.001481909158315892</v>
+        <v>0.001595294677002861</v>
       </c>
     </row>
     <row r="87" spans="1:2">
       <c r="A87">
-        <v>699.5424242424242</v>
+        <v>691.0151515151515</v>
       </c>
       <c r="B87">
-        <v>0.001461023442126762</v>
+        <v>0.001574271709285973</v>
       </c>
     </row>
     <row r="88" spans="1:2">
       <c r="A88">
-        <v>707.6393939393939</v>
+        <v>699.0212121212121</v>
       </c>
       <c r="B88">
-        <v>0.001440667398165869</v>
+        <v>0.001553763203034644</v>
       </c>
     </row>
     <row r="89" spans="1:2">
       <c r="A89">
-        <v>715.7363636363636</v>
+        <v>707.0272727272727</v>
       </c>
       <c r="B89">
-        <v>0.001420821760896863</v>
+        <v>0.001533750890185145</v>
       </c>
     </row>
     <row r="90" spans="1:2">
       <c r="A90">
-        <v>723.8333333333334</v>
+        <v>715.0333333333333</v>
       </c>
       <c r="B90">
-        <v>0.001401468172932123</v>
+        <v>0.001514217348481232</v>
       </c>
     </row>
     <row r="91" spans="1:2">
       <c r="A91">
-        <v>731.9303030303031</v>
+        <v>723.0393939393939</v>
       </c>
       <c r="B91">
-        <v>0.001382589132662983</v>
+        <v>0.001495145953388581</v>
       </c>
     </row>
     <row r="92" spans="1:2">
       <c r="A92">
-        <v>740.0272727272727</v>
+        <v>731.0454545454545</v>
       </c>
       <c r="B92">
-        <v>0.001364167945449245</v>
+        <v>0.001476520833239256</v>
       </c>
     </row>
     <row r="93" spans="1:2">
       <c r="A93">
-        <v>748.1242424242424</v>
+        <v>739.0515151515151</v>
       </c>
       <c r="B93">
-        <v>0.001346188678090202</v>
+        <v>0.00145832682735662</v>
       </c>
     </row>
     <row r="94" spans="1:2">
       <c r="A94">
-        <v>756.2212121212121</v>
+        <v>747.0575757575757</v>
       </c>
       <c r="B94">
-        <v>0.001328636116323822</v>
+        <v>0.001440549446932866</v>
       </c>
     </row>
     <row r="95" spans="1:2">
       <c r="A95">
-        <v>764.3181818181819</v>
+        <v>755.0636363636363</v>
       </c>
       <c r="B95">
-        <v>0.001311495725122791</v>
+        <v>0.001423174838450966</v>
       </c>
     </row>
     <row r="96" spans="1:2">
       <c r="A96">
-        <v>772.4151515151515</v>
+        <v>763.0696969696969</v>
       </c>
       <c r="B96">
-        <v>0.00129475361157598</v>
+        <v>0.001406189749460629</v>
       </c>
     </row>
     <row r="97" spans="1:2">
       <c r="A97">
-        <v>780.5121212121212</v>
+        <v>771.0757575757575</v>
       </c>
       <c r="B97">
-        <v>0.001278396490161965</v>
+        <v>0.001389581496533911</v>
       </c>
     </row>
     <row r="98" spans="1:2">
       <c r="A98">
-        <v>788.6090909090909</v>
+        <v>779.0818181818181</v>
       </c>
       <c r="B98">
-        <v>0.001262411650237472</v>
+        <v>0.00137333793524071</v>
       </c>
     </row>
     <row r="99" spans="1:2">
       <c r="A99">
-        <v>796.7060606060606</v>
+        <v>787.0878787878788</v>
       </c>
       <c r="B99">
-        <v>0.001246786925578432</v>
+        <v>0.001357447431997586</v>
       </c>
     </row>
     <row r="100" spans="1:2">
       <c r="A100">
-        <v>804.8030303030304</v>
+        <v>795.0939393939394</v>
       </c>
       <c r="B100">
-        <v>0.001231510665824734</v>
+        <v>0.00134189883765535</v>
       </c>
     </row>
     <row r="101" spans="1:2">
       <c r="A101">
-        <v>812.9</v>
+        <v>803.1</v>
       </c>
       <c r="B101">
-        <v>0.001216571709691934</v>
+        <v>0.00132668146270177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>